<commit_message>
Expand pairing map to 3 ranked matches per collection
Restructure pairs_with into match_1/match_2/match_3 (best-fit first).
Preserve reviewed match_1; add two ranked alternates per pairable row
so the cross/up-sell injector always has multiple in-stock sources.
Validates every target is published, has products, and is distinct
(no self/duplicate within a row).
</commit_message>
<xml_diff>
--- a/phoenix_collections_pairing_map_FILLED.xlsx
+++ b/phoenix_collections_pairing_map_FILLED.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F224"/>
+  <dimension ref="A1:H224"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -480,12 +480,22 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>pairs_with (you fill)</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>notes (you fill)</t>
+          <t>match_1</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>match_2</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>match_3</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>notes</t>
         </is>
       </c>
     </row>
@@ -509,7 +519,17 @@
           <t>wierookhouders-en-accessoires</t>
         </is>
       </c>
-      <c r="F2" s="2" t="n"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>alle-wierook</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>engel-producten</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -531,7 +551,17 @@
           <t>alle-kristallen-klankschalen</t>
         </is>
       </c>
-      <c r="F3" s="2" t="n"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>sound-healing-instrumenten</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>accessoires-metalen-klankschalen</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -553,7 +583,17 @@
           <t>alle-metalen-klankschalen</t>
         </is>
       </c>
-      <c r="F4" s="2" t="n"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>sound-healing-instrumenten</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>accessoires-kristallen-klankschalen</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -575,7 +615,17 @@
           <t>wierookhouders-en-accessoires</t>
         </is>
       </c>
-      <c r="F5" s="2" t="n"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>alle-wierook</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>masala-en-ayurvedische-wierook</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -597,7 +647,17 @@
           <t>klein-meubilair-en-decoratie</t>
         </is>
       </c>
-      <c r="F6" s="2" t="n"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>boeddha-beelden</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>hindoe-beelden</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -619,7 +679,17 @@
           <t>olieverdampers-en-geurstenen</t>
         </is>
       </c>
-      <c r="F7" s="2" t="n"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>biologische-etherische-olie</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>aroma-diffusers</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -641,7 +711,17 @@
           <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
-      <c r="F8" s="2" t="n"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>geurkaarsen</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>zoutkristal-kaarshouders</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -663,7 +743,17 @@
           <t>accessoires-kristallen-klankschalen</t>
         </is>
       </c>
-      <c r="F9" s="2" t="n"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>sound-healing-instrumenten</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>alle-metalen-klankschalen</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -685,7 +775,17 @@
           <t>meditatie-omslagdoeken-en-accessoires</t>
         </is>
       </c>
-      <c r="F10" s="2" t="n"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>meditatiematten-en-meditatiesets</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>meditatiebankjes</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -707,7 +807,17 @@
           <t>accessoires-metalen-klankschalen</t>
         </is>
       </c>
-      <c r="F11" s="2" t="n"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>sound-healing-instrumenten</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>alle-kristallen-klankschalen</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -729,7 +839,17 @@
           <t>sieraden-opbergdozen-en-tasjes</t>
         </is>
       </c>
-      <c r="F12" s="2" t="n"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>edelsteen-armbanden</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>edelsteen-hangers-gepolijst</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -751,7 +871,17 @@
           <t>wierookhouders-en-accessoires</t>
         </is>
       </c>
-      <c r="F13" s="2" t="n"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>houtskool-en-houtkoolbranders</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>wierookharsen-en-wierookkruiden</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -773,7 +903,17 @@
           <t>sieraden-opbergdozen-en-tasjes</t>
         </is>
       </c>
-      <c r="F14" s="2" t="n"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>alle-sieraden</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>edelsteen-armbanden</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -795,7 +935,17 @@
           <t>sieraden-opbergdozen-en-tasjes</t>
         </is>
       </c>
-      <c r="F15" s="2" t="n"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>alle-sieraden</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>hangers-metaal</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -817,7 +967,17 @@
           <t>alle-etherische-olien</t>
         </is>
       </c>
-      <c r="F16" s="2" t="n"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>olieverdampers-en-geurstenen</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>interieur-geurproducten</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="n"/>
     </row>
     <row r="17" customFormat="1" s="5">
       <c r="A17" s="4" t="inlineStr">
@@ -839,7 +999,17 @@
           <t>olieverdampers-en-geurstenen</t>
         </is>
       </c>
-      <c r="F17" s="4" t="n"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>aromafume-geurproducten</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>aromafume-wierookblokjes-non-toxic</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -861,7 +1031,17 @@
           <t>olieverdampers-en-geurstenen</t>
         </is>
       </c>
-      <c r="F18" s="2" t="n"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>aromafume-alle-producten</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>interieur-geurproducten</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -883,7 +1063,17 @@
           <t>wierookhouders-en-accessoires</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>aromafume-alle-producten</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>alle-wierook</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>incense -&gt; needs holder/burner</t>
         </is>
@@ -909,7 +1099,17 @@
           <t>bach-producten-elixirs-co</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>biologische-ontspanningsproducten</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>lichaamsverzorging-producten</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>Bach flowers &lt;-&gt; Bach elixirs</t>
         </is>
@@ -935,7 +1135,17 @@
           <t>bach-bloesem-producten</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>biologische-ontspanningsproducten</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>lichaamsverzorging-producten</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>Bach elixirs &lt;-&gt; Bach flowers</t>
         </is>
@@ -961,7 +1171,17 @@
           <t>wierookhouders-en-accessoires</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>wierookkegels</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>alle-wierook</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>backflow burners/cones -&gt; incense accessories</t>
         </is>
@@ -987,7 +1207,17 @@
           <t>lichaamsverzorging-producten</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>biologische-lichaamsverzorging</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>haarverzorging</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>bath/soap -&gt; body care</t>
         </is>
@@ -1013,7 +1243,17 @@
           <t>klein-meubilair-en-decoratie</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>kathas-altaar-en-deurkleden</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>tibetaanse-gebedsvlaggen</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>wall hangings -&gt; decor</t>
         </is>
@@ -1039,7 +1279,7 @@
         </is>
       </c>
       <c r="E25" s="3" t="n"/>
-      <c r="F25" s="3" t="n"/>
+      <c r="H25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1061,7 +1301,17 @@
           <t>sieraden-opbergdozen-en-tasjes</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>edelsteen-hangers-gepolijst</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>alle-sieraden</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>pendants -&gt; storage</t>
         </is>
@@ -1087,7 +1337,7 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>merch bucket - no logical pair</t>
         </is>
@@ -1113,7 +1363,17 @@
           <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>alle-kaarsen</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>dinerkaarsen-en-stompkaarsen</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>candles -&gt; holders/lights</t>
         </is>
@@ -1139,7 +1399,17 @@
           <t>olieverdampers-en-geurstenen</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>alle-etherische-olien</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>aroma-diffusers</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>oils -&gt; diffuser</t>
         </is>
@@ -1165,7 +1435,17 @@
           <t>lichaamsverzorging-producten</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>bad-douche-en-zeep</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>biologische-ontspanningsproducten</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>organic -&gt; body care</t>
         </is>
@@ -1191,7 +1471,17 @@
           <t>meditatie-omslagdoeken-en-accessoires</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>alle-meditatiekussens</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>meditatiekussens-rond-biologisch</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>cushion -&gt; meditation accessories</t>
         </is>
@@ -1217,7 +1507,17 @@
           <t>biologische-thee</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>lichaamsverzorging-producten</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>bach-bloesem-producten</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>relaxation -&gt; organic tea</t>
         </is>
@@ -1243,7 +1543,7 @@
         </is>
       </c>
       <c r="E33" s="3" t="n"/>
-      <c r="F33" s="3" t="n"/>
+      <c r="H33" s="3" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1265,7 +1565,17 @@
           <t>thee-accessoires</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>thee-alle-producten</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>thee-shoti-maa-biologisch</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>tea -&gt; tea accessories</t>
         </is>
@@ -1291,7 +1601,17 @@
           <t>yogamatten-en-handdoeken</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>yoga-welzijn</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>biologische-meditatiekussens</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
         <is>
           <t>organic yoga -&gt; mats</t>
         </is>
@@ -1317,7 +1637,17 @@
           <t>pendel-accessoires</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>pendels-voor-professionals</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>pendels-van-mineralen-hout-en-rudraksha</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>dowsing tools -&gt; pendulum accessories</t>
         </is>
@@ -1343,7 +1673,17 @@
           <t>levensboom-producten</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>sieraden-bloem-des-levens</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>klein-meubilair-en-decoratie</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>flower of life &lt;-&gt; tree of life (sacred geometry)</t>
         </is>
@@ -1369,7 +1709,17 @@
           <t>klein-meubilair-en-decoratie</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>alle-beelden</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>hindoe-beelden</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t>statues -&gt; furniture/decor</t>
         </is>
@@ -1395,7 +1745,7 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="F39" s="2" t="inlineStr">
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>test collection - no logical pair</t>
         </is>
@@ -1421,7 +1771,17 @@
           <t>chakra-producten</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>trommelstenen</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>wicca-en-tarot</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
         <is>
           <t>mineral sets -&gt; chakra range</t>
         </is>
@@ -1447,7 +1807,17 @@
           <t>chakra-en-wicca-mineraalsets</t>
         </is>
       </c>
-      <c r="F41" s="2" t="inlineStr">
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>sieraden-chakras</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>meditatiekussens-en-matten-chakras</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>chakra -&gt; mineral sets</t>
         </is>
@@ -1473,7 +1843,17 @@
           <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>alle-kaarsen</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>zoutkristal-kaarshouders</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
         <is>
           <t>candles -&gt; holders/lights</t>
         </is>
@@ -1499,7 +1879,17 @@
           <t>sieraden-opbergdozen-en-tasjes</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr">
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>alle-sieraden</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>armbanden-edelsteen-aa</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
         <is>
           <t>jewelry -&gt; storage</t>
         </is>
@@ -1525,7 +1915,17 @@
           <t>mineralen-decoratie-producten</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>edelsteen-piramides-obelisk</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>ruwe-onbewerkte-mineralen</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
         <is>
           <t>gemstone spheres -&gt; mineral decor</t>
         </is>
@@ -1551,7 +1951,17 @@
           <t>seleniet-producten</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr">
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>zoutlampen-en-meer</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>mineralen-decoratie-producten</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
         <is>
           <t>selenite lamps -&gt; selenite range</t>
         </is>
@@ -1577,7 +1987,17 @@
           <t>engel-producten</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>mineralen-decoratie-producten</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>engelen-beelden</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
         <is>
           <t>gemstone angels -&gt; angel range</t>
         </is>
@@ -1603,7 +2023,17 @@
           <t>sieraden-opbergdozen-en-tasjes</t>
         </is>
       </c>
-      <c r="F47" s="2" t="inlineStr">
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>hangers-edelsteen-geboord</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>alle-sieraden</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
         <is>
           <t>pendants -&gt; storage</t>
         </is>
@@ -1629,7 +2059,17 @@
           <t>sieraden-opbergdozen-en-tasjes</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>edelsteen-hangers-gepolijst</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>alle-sieraden</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
         <is>
           <t>pendants -&gt; storage</t>
         </is>
@@ -1655,7 +2095,17 @@
           <t>sieraden-opbergdozen-en-tasjes</t>
         </is>
       </c>
-      <c r="F49" s="2" t="inlineStr">
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>alle-sieraden</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>oorbellen</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
         <is>
           <t>jewelry -&gt; storage</t>
         </is>
@@ -1681,7 +2131,17 @@
           <t>mineralen-decoratie-producten</t>
         </is>
       </c>
-      <c r="F50" s="2" t="inlineStr">
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>edelsteen-bollen</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>seleniet-producten</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
         <is>
           <t>gemstone shapes -&gt; mineral decor</t>
         </is>
@@ -1707,7 +2167,17 @@
           <t>sieraden-opbergdozen-en-tasjes</t>
         </is>
       </c>
-      <c r="F51" s="2" t="inlineStr">
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>alle-sieraden</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>ringen</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
         <is>
           <t>jewelry -&gt; storage</t>
         </is>
@@ -1733,7 +2203,17 @@
           <t>lichaamsverzorging-producten</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr">
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>haarverzorging</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>bad-douche-en-zeep</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
         <is>
           <t>ayurvedic brand -&gt; body care</t>
         </is>
@@ -1759,7 +2239,17 @@
           <t>engelen-beelden</t>
         </is>
       </c>
-      <c r="F53" s="2" t="inlineStr">
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>sieraden-engelen</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>edelsteen-engelen</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
         <is>
           <t>angel range -&gt; angel statues</t>
         </is>
@@ -1785,7 +2275,17 @@
           <t>klein-meubilair-en-decoratie</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>engel-producten</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>alle-beelden</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
         <is>
           <t>statues -&gt; furniture/decor</t>
         </is>
@@ -1811,7 +2311,17 @@
           <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
-      <c r="F55" s="2" t="inlineStr">
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>alle-kaarsen</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>engel-producten</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
         <is>
           <t>candles -&gt; holders/lights</t>
         </is>
@@ -1837,7 +2347,17 @@
           <t>feng-shui-producten</t>
         </is>
       </c>
-      <c r="F56" s="2" t="inlineStr">
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>orgoniet-producten</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>mineralen-decoratie-producten</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
         <is>
           <t>crystal feng shui &lt;-&gt; feng shui</t>
         </is>
@@ -1863,7 +2383,17 @@
           <t>feng-shui-kristalproducten</t>
         </is>
       </c>
-      <c r="F57" s="2" t="inlineStr">
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>orgoniet-producten</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>mineralen-decoratie-producten</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
         <is>
           <t>feng shui &lt;-&gt; crystal feng shui</t>
         </is>
@@ -1889,7 +2419,17 @@
           <t>olieverdampers-en-geurstenen</t>
         </is>
       </c>
-      <c r="F58" s="2" t="inlineStr">
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>alle-etherische-olien</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>fiore-doriente-wierook</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
         <is>
           <t>oils -&gt; diffuser</t>
         </is>
@@ -1915,7 +2455,17 @@
           <t>wierookhouders-en-accessoires</t>
         </is>
       </c>
-      <c r="F59" s="2" t="n"/>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>alle-wierook</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>fiore-doriente-essentiele-olien</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -1937,7 +2487,17 @@
           <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
-      <c r="F60" s="2" t="inlineStr">
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>alle-kaarsen</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>interieur-geurproducten</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
         <is>
           <t>candles -&gt; holders/lights</t>
         </is>
@@ -1963,7 +2523,7 @@
         </is>
       </c>
       <c r="E61" s="3" t="n"/>
-      <c r="F61" s="3" t="n"/>
+      <c r="H61" s="3" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -1985,7 +2545,17 @@
           <t>lichaamsverzorging-producten</t>
         </is>
       </c>
-      <c r="F62" s="2" t="inlineStr">
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>bad-douche-en-zeep</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>biologische-lichaamsverzorging</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
         <is>
           <t>face care -&gt; body care</t>
         </is>
@@ -2011,7 +2581,7 @@
         </is>
       </c>
       <c r="E63" s="3" t="n"/>
-      <c r="F63" s="3" t="n"/>
+      <c r="H63" s="3" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -2033,7 +2603,17 @@
           <t>sound-healing-instrumenten</t>
         </is>
       </c>
-      <c r="F64" s="2" t="inlineStr">
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>alle-metalen-klankschalen</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>stemvorken</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
         <is>
           <t>gongs -&gt; sound healing range</t>
         </is>
@@ -2059,7 +2639,17 @@
           <t>lichaamsverzorging-producten</t>
         </is>
       </c>
-      <c r="F65" s="2" t="inlineStr">
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>bad-douche-en-zeep</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>gezichtsverzorging</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
         <is>
           <t>hair care -&gt; body care</t>
         </is>
@@ -2085,7 +2675,17 @@
           <t>sieraden-opbergdozen-en-tasjes</t>
         </is>
       </c>
-      <c r="F66" s="2" t="inlineStr">
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>edelsteen-hangers-gepolijst</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>alle-sieraden</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
         <is>
           <t>pendants -&gt; storage</t>
         </is>
@@ -2111,7 +2711,17 @@
           <t>sieraden-opbergdozen-en-tasjes</t>
         </is>
       </c>
-      <c r="F67" s="2" t="inlineStr">
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>edelsteen-hangers-gepolijst</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>alle-sieraden</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
         <is>
           <t>pendants -&gt; storage</t>
         </is>
@@ -2137,7 +2747,17 @@
           <t>sieraden-opbergdozen-en-tasjes</t>
         </is>
       </c>
-      <c r="F68" s="2" t="inlineStr">
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>hangers-overig</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>alle-sieraden</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
         <is>
           <t>pendants -&gt; storage</t>
         </is>
@@ -2163,7 +2783,17 @@
           <t>sieraden-opbergdozen-en-tasjes</t>
         </is>
       </c>
-      <c r="F69" s="2" t="inlineStr">
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>hangers-metaal</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>alle-sieraden</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
         <is>
           <t>pendants -&gt; storage</t>
         </is>
@@ -2189,7 +2819,17 @@
           <t>lichaamsverzorging-producten</t>
         </is>
       </c>
-      <c r="F70" s="2" t="inlineStr">
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>gezichtsverzorging</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>haarverzorging</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
         <is>
           <t>care brand -&gt; body care</t>
         </is>
@@ -2215,7 +2855,17 @@
           <t>lichaamsverzorging-producten</t>
         </is>
       </c>
-      <c r="F71" s="2" t="inlineStr">
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>bad-douche-en-zeep</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>gezichtsverzorging</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
         <is>
           <t>brand -&gt; body care</t>
         </is>
@@ -2241,7 +2891,17 @@
           <t>klein-meubilair-en-decoratie</t>
         </is>
       </c>
-      <c r="F72" s="2" t="inlineStr">
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>alle-beelden</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>boeddha-beelden</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
         <is>
           <t>statues -&gt; furniture/decor</t>
         </is>
@@ -2267,7 +2927,17 @@
           <t>lichaamsverzorging-producten</t>
         </is>
       </c>
-      <c r="F73" s="2" t="inlineStr">
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>bad-douche-en-zeep</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>parfums-eau-de-toilettes</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
         <is>
           <t>care brand -&gt; body care</t>
         </is>
@@ -2293,7 +2963,7 @@
         </is>
       </c>
       <c r="E74" s="3" t="n"/>
-      <c r="F74" s="3" t="n"/>
+      <c r="H74" s="3" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
@@ -2315,7 +2985,7 @@
         </is>
       </c>
       <c r="E75" s="3" t="n"/>
-      <c r="F75" s="3" t="n"/>
+      <c r="H75" s="3" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -2337,7 +3007,17 @@
           <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
-      <c r="F76" s="2" t="inlineStr">
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>alle-kaarsen</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>votiefkaarsen</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
         <is>
           <t>candles -&gt; holders/lights</t>
         </is>
@@ -2363,7 +3043,17 @@
           <t>wierookharsen-en-wierookkruiden</t>
         </is>
       </c>
-      <c r="F77" s="2" t="inlineStr">
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>alle-wierook</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>witte-salie-en-smudges</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
         <is>
           <t>charcoal -&gt; resins to burn</t>
         </is>
@@ -2389,7 +3079,17 @@
           <t>stickers</t>
         </is>
       </c>
-      <c r="F78" s="2" t="inlineStr">
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>raamstickers</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>notitieboeken-en-meer</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
         <is>
           <t>mandala stickers -&gt; stickers</t>
         </is>
@@ -2415,7 +3115,17 @@
           <t>olieverdampers-en-geurstenen</t>
         </is>
       </c>
-      <c r="F79" s="2" t="inlineStr">
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>geurkaarsen</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>alle-etherische-olien</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
         <is>
           <t>interior scent -&gt; diffuser</t>
         </is>
@@ -2441,7 +3151,17 @@
           <t>wierookhouders-en-accessoires</t>
         </is>
       </c>
-      <c r="F80" s="2" t="inlineStr">
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>alle-wierook</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>palo-santo-alle-producten</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
         <is>
           <t>incense -&gt; needs holder</t>
         </is>
@@ -2467,7 +3187,7 @@
         </is>
       </c>
       <c r="E81" s="3" t="n"/>
-      <c r="F81" s="3" t="n"/>
+      <c r="H81" s="3" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -2489,7 +3209,17 @@
           <t>klein-meubilair-en-decoratie</t>
         </is>
       </c>
-      <c r="F82" s="2" t="inlineStr">
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>feng-shui-producten</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>zoutlampen-en-meer</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
         <is>
           <t>fountains -&gt; decor</t>
         </is>
@@ -2515,7 +3245,17 @@
           <t>rituele-voorwerpen</t>
         </is>
       </c>
-      <c r="F83" s="2" t="inlineStr">
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>banners-wandkleden-en-strandlakens</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>klein-meubilair-en-decoratie</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
         <is>
           <t>altar cloths -&gt; ritual objects</t>
         </is>
@@ -2541,7 +3281,17 @@
           <t>lichaamsverzorging-producten</t>
         </is>
       </c>
-      <c r="F84" s="2" t="inlineStr">
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>bad-douche-en-zeep</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>gezichtsverzorging</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
         <is>
           <t>oral care -&gt; body care</t>
         </is>
@@ -2567,7 +3317,17 @@
           <t>sieraden-opbergdozen-en-tasjes</t>
         </is>
       </c>
-      <c r="F85" s="2" t="inlineStr">
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>alle-sieraden</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>malas-en-mala-tasjes</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
         <is>
           <t>jewelry -&gt; storage</t>
         </is>
@@ -2593,7 +3353,17 @@
           <t>sound-healing-instrumenten</t>
         </is>
       </c>
-      <c r="F86" s="2" t="inlineStr">
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>stemvorken</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>alle-metalen-klankschalen</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
         <is>
           <t>chimes/bars -&gt; sound healing range</t>
         </is>
@@ -2619,7 +3389,17 @@
           <t>accessoires-metalen-klankschalen</t>
         </is>
       </c>
-      <c r="F87" s="2" t="inlineStr">
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>alle-metalen-klankschalen</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>sound-healing-instrumenten</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
         <is>
           <t>metal bowl -&gt; accessories</t>
         </is>
@@ -2645,7 +3425,17 @@
           <t>accessoires-metalen-klankschalen</t>
         </is>
       </c>
-      <c r="F88" s="2" t="inlineStr">
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>alle-metalen-klankschalen</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>chakra-producten</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
         <is>
           <t>metal bowl -&gt; accessories</t>
         </is>
@@ -2671,7 +3461,17 @@
           <t>accessoires-metalen-klankschalen</t>
         </is>
       </c>
-      <c r="F89" s="2" t="inlineStr">
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>alle-metalen-klankschalen</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>sound-healing-instrumenten</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
         <is>
           <t>metal bowl -&gt; accessories</t>
         </is>
@@ -2697,7 +3497,17 @@
           <t>accessoires-metalen-klankschalen</t>
         </is>
       </c>
-      <c r="F90" s="2" t="inlineStr">
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>alle-metalen-klankschalen</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>sound-healing-instrumenten</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
         <is>
           <t>metal bowl -&gt; accessories</t>
         </is>
@@ -2723,7 +3533,7 @@
         </is>
       </c>
       <c r="E91" s="3" t="n"/>
-      <c r="F91" s="3" t="n"/>
+      <c r="H91" s="3" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -2745,7 +3555,17 @@
           <t>accessoires-metalen-klankschalen</t>
         </is>
       </c>
-      <c r="F92" s="2" t="inlineStr">
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>alle-metalen-klankschalen</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>sound-healing-instrumenten</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
         <is>
           <t>metal bowl -&gt; accessories</t>
         </is>
@@ -2771,7 +3591,17 @@
           <t>accessoires-metalen-klankschalen</t>
         </is>
       </c>
-      <c r="F93" s="2" t="inlineStr">
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>alle-metalen-klankschalen</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>sound-healing-instrumenten</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
         <is>
           <t>metal bowl -&gt; accessories</t>
         </is>
@@ -2797,7 +3627,17 @@
           <t>accessoires-metalen-klankschalen</t>
         </is>
       </c>
-      <c r="F94" s="2" t="inlineStr">
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>alle-metalen-klankschalen</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>sound-healing-instrumenten</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
         <is>
           <t>metal bowl -&gt; accessories</t>
         </is>
@@ -2823,7 +3663,17 @@
           <t>accessoires-metalen-klankschalen</t>
         </is>
       </c>
-      <c r="F95" s="2" t="inlineStr">
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>alle-metalen-klankschalen</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>sound-healing-instrumenten</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
         <is>
           <t>metal bowl -&gt; accessories</t>
         </is>
@@ -2849,7 +3699,17 @@
           <t>accessoires-metalen-klankschalen</t>
         </is>
       </c>
-      <c r="F96" s="2" t="inlineStr">
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>alle-metalen-klankschalen</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>sound-healing-instrumenten</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
         <is>
           <t>metal bowl -&gt; accessories</t>
         </is>
@@ -2875,7 +3735,17 @@
           <t>accessoires-metalen-klankschalen</t>
         </is>
       </c>
-      <c r="F97" s="2" t="inlineStr">
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>alle-metalen-klankschalen</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>sound-healing-instrumenten</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
         <is>
           <t>metal bowl -&gt; accessories</t>
         </is>
@@ -2901,7 +3771,17 @@
           <t>accessoires-metalen-klankschalen</t>
         </is>
       </c>
-      <c r="F98" s="2" t="inlineStr">
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>alle-metalen-klankschalen</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>sound-healing-instrumenten</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr">
         <is>
           <t>metal bowl -&gt; accessories</t>
         </is>
@@ -2927,7 +3807,17 @@
           <t>accessoires-metalen-klankschalen</t>
         </is>
       </c>
-      <c r="F99" s="2" t="inlineStr">
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>alle-metalen-klankschalen</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>sound-healing-instrumenten</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="inlineStr">
         <is>
           <t>metal bowl -&gt; accessories</t>
         </is>
@@ -2953,7 +3843,17 @@
           <t>accessoires-metalen-klankschalen</t>
         </is>
       </c>
-      <c r="F100" s="2" t="inlineStr">
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>alle-metalen-klankschalen</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>sound-healing-instrumenten</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="inlineStr">
         <is>
           <t>metal bowl -&gt; accessories</t>
         </is>
@@ -2979,7 +3879,17 @@
           <t>accessoires-metalen-klankschalen</t>
         </is>
       </c>
-      <c r="F101" s="2" t="inlineStr">
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>alle-metalen-klankschalen</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>sound-healing-instrumenten</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr">
         <is>
           <t>metal bowl -&gt; accessories</t>
         </is>
@@ -3005,7 +3915,17 @@
           <t>alle-beelden</t>
         </is>
       </c>
-      <c r="F102" s="2" t="inlineStr">
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>mineralen-decoratie-producten</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>kamerfonteinen</t>
+        </is>
+      </c>
+      <c r="H102" s="2" t="inlineStr">
         <is>
           <t>small furniture &lt;-&gt; statues</t>
         </is>
@@ -3031,7 +3951,17 @@
           <t>accessoires-kristallen-klankschalen</t>
         </is>
       </c>
-      <c r="F103" s="2" t="inlineStr">
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>alle-kristallen-klankschalen</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>sound-healing-instrumenten</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="inlineStr">
         <is>
           <t>crystal bowl -&gt; accessories</t>
         </is>
@@ -3057,7 +3987,17 @@
           <t>accessoires-kristallen-klankschalen</t>
         </is>
       </c>
-      <c r="F104" s="2" t="inlineStr">
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>alle-kristallen-klankschalen</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>sound-healing-instrumenten</t>
+        </is>
+      </c>
+      <c r="H104" s="2" t="inlineStr">
         <is>
           <t>crystal bowl -&gt; accessories</t>
         </is>
@@ -3083,7 +4023,17 @@
           <t>accessoires-kristallen-klankschalen</t>
         </is>
       </c>
-      <c r="F105" s="2" t="inlineStr">
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>alle-kristallen-klankschalen</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>sound-healing-instrumenten</t>
+        </is>
+      </c>
+      <c r="H105" s="2" t="inlineStr">
         <is>
           <t>crystal bowl -&gt; accessories</t>
         </is>
@@ -3109,7 +4059,17 @@
           <t>accessoires-kristallen-klankschalen</t>
         </is>
       </c>
-      <c r="F106" s="2" t="inlineStr">
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>alle-kristallen-klankschalen</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>sound-healing-instrumenten</t>
+        </is>
+      </c>
+      <c r="H106" s="2" t="inlineStr">
         <is>
           <t>crystal bowl -&gt; accessories</t>
         </is>
@@ -3135,7 +4095,17 @@
           <t>lichaamsverzorging-producten</t>
         </is>
       </c>
-      <c r="F107" s="2" t="inlineStr">
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>bad-douche-en-zeep</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>biologische-ontspanningsproducten</t>
+        </is>
+      </c>
+      <c r="H107" s="2" t="inlineStr">
         <is>
           <t>lavender -&gt; body care</t>
         </is>
@@ -3161,7 +4131,17 @@
           <t>bad-douche-en-zeep</t>
         </is>
       </c>
-      <c r="F108" s="2" t="inlineStr">
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>lichaamsverzorging-producten</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>parfums-eau-de-toilettes</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="inlineStr">
         <is>
           <t>soap brand -&gt; bath/soap</t>
         </is>
@@ -3187,7 +4167,17 @@
           <t>lichaamsverzorging-producten</t>
         </is>
       </c>
-      <c r="F109" s="2" t="inlineStr">
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>bad-douche-en-zeep</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>gezichtsverzorging</t>
+        </is>
+      </c>
+      <c r="H109" s="2" t="inlineStr">
         <is>
           <t>care brand -&gt; body care</t>
         </is>
@@ -3213,7 +4203,17 @@
           <t>bloem-des-levens-producten</t>
         </is>
       </c>
-      <c r="F110" s="2" t="inlineStr">
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>klein-meubilair-en-decoratie</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>sieraden-bloem-des-levens</t>
+        </is>
+      </c>
+      <c r="H110" s="2" t="inlineStr">
         <is>
           <t>tree of life &lt;-&gt; flower of life (sacred geometry)</t>
         </is>
@@ -3239,7 +4239,17 @@
           <t>bad-douche-en-zeep</t>
         </is>
       </c>
-      <c r="F111" s="2" t="inlineStr">
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>biologische-lichaamsverzorging</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>gezichtsverzorging</t>
+        </is>
+      </c>
+      <c r="H111" s="2" t="inlineStr">
         <is>
           <t>body care -&gt; bath/soap</t>
         </is>
@@ -3265,7 +4275,7 @@
         </is>
       </c>
       <c r="E112" s="3" t="n"/>
-      <c r="F112" s="3" t="n"/>
+      <c r="H112" s="3" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -3287,7 +4297,17 @@
           <t>alle-kaarsen</t>
         </is>
       </c>
-      <c r="F113" s="2" t="inlineStr">
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>sfeerlichten-en-lantaarns</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>waxinelichtjes</t>
+        </is>
+      </c>
+      <c r="H113" s="2" t="inlineStr">
         <is>
           <t>tealight holders -&gt; need candles</t>
         </is>
@@ -3313,7 +4333,7 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="F114" s="2" t="inlineStr">
+      <c r="H114" s="2" t="inlineStr">
         <is>
           <t>merch bucket - no logical pair</t>
         </is>
@@ -3339,7 +4359,7 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="F115" s="2" t="inlineStr">
+      <c r="H115" s="2" t="inlineStr">
         <is>
           <t>merch bucket - no logical pair</t>
         </is>
@@ -3365,7 +4385,17 @@
           <t>postkaarten</t>
         </is>
       </c>
-      <c r="F116" s="2" t="inlineStr">
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>notitieboeken-en-meer</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>stickers</t>
+        </is>
+      </c>
+      <c r="H116" s="2" t="inlineStr">
         <is>
           <t>small gifts -&gt; postcards</t>
         </is>
@@ -3391,7 +4421,17 @@
           <t>sieraden-opbergdozen-en-tasjes</t>
         </is>
       </c>
-      <c r="F117" s="2" t="inlineStr">
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>kettingen-en-malas</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>alle-sieraden</t>
+        </is>
+      </c>
+      <c r="H117" s="2" t="inlineStr">
         <is>
           <t>jewelry -&gt; storage</t>
         </is>
@@ -3417,7 +4457,17 @@
           <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
-      <c r="F118" s="2" t="inlineStr">
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>alle-kaarsen</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>wicca-en-tarot</t>
+        </is>
+      </c>
+      <c r="H118" s="2" t="inlineStr">
         <is>
           <t>candles -&gt; holders/lights</t>
         </is>
@@ -3443,7 +4493,17 @@
           <t>wierookhouders-en-accessoires</t>
         </is>
       </c>
-      <c r="F119" s="2" t="inlineStr">
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>alle-wierook</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>nag-champa-en-satya-wierook</t>
+        </is>
+      </c>
+      <c r="H119" s="2" t="inlineStr">
         <is>
           <t>incense -&gt; needs holder</t>
         </is>
@@ -3469,7 +4529,17 @@
           <t>massageolie</t>
         </is>
       </c>
-      <c r="F120" s="2" t="inlineStr">
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>meridiaankogels</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>lichaamsverzorging-producten</t>
+        </is>
+      </c>
+      <c r="H120" s="2" t="inlineStr">
         <is>
           <t>massage tools -&gt; massage oil</t>
         </is>
@@ -3495,7 +4565,17 @@
           <t>massage-hulpmiddelen</t>
         </is>
       </c>
-      <c r="F121" s="2" t="inlineStr">
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>lichaamsverzorging-producten</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>biologische-ontspanningsproducten</t>
+        </is>
+      </c>
+      <c r="H121" s="2" t="inlineStr">
         <is>
           <t>massage oil -&gt; massage tools</t>
         </is>
@@ -3521,7 +4601,7 @@
         </is>
       </c>
       <c r="E122" s="3" t="n"/>
-      <c r="F122" s="3" t="n"/>
+      <c r="H122" s="3" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -3543,7 +4623,17 @@
           <t>watervitalisering-alle-producten</t>
         </is>
       </c>
-      <c r="F123" s="2" t="inlineStr">
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>watervitalisering-natures-design</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>watervitalisering-vitajuwel</t>
+        </is>
+      </c>
+      <c r="H123" s="2" t="inlineStr">
         <is>
           <t>gemstone bottles -&gt; water vitalization</t>
         </is>
@@ -3569,7 +4659,17 @@
           <t>alle-meditatiekussens</t>
         </is>
       </c>
-      <c r="F124" s="2" t="inlineStr">
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>meditatiebankjes</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>sjaals-en-pashminas</t>
+        </is>
+      </c>
+      <c r="H124" s="2" t="inlineStr">
         <is>
           <t>accessories -&gt; all cushions</t>
         </is>
@@ -3595,7 +4695,17 @@
           <t>meditatie-omslagdoeken-en-accessoires</t>
         </is>
       </c>
-      <c r="F125" s="2" t="inlineStr">
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>alle-meditatiekussens</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>meditatiematten-en-meditatiesets</t>
+        </is>
+      </c>
+      <c r="H125" s="2" t="inlineStr">
         <is>
           <t>benches -&gt; meditation accessories</t>
         </is>
@@ -3621,7 +4731,17 @@
           <t>meditatie-omslagdoeken-en-accessoires</t>
         </is>
       </c>
-      <c r="F126" s="2" t="inlineStr">
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>alle-meditatiekussens</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>chakra-producten</t>
+        </is>
+      </c>
+      <c r="H126" s="2" t="inlineStr">
         <is>
           <t>cushion -&gt; meditation accessories</t>
         </is>
@@ -3647,7 +4767,17 @@
           <t>meditatie-omslagdoeken-en-accessoires</t>
         </is>
       </c>
-      <c r="F127" s="2" t="inlineStr">
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>alle-meditatiekussens</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>meditatiekussens-rond</t>
+        </is>
+      </c>
+      <c r="H127" s="2" t="inlineStr">
         <is>
           <t>cushion -&gt; meditation accessories</t>
         </is>
@@ -3673,7 +4803,17 @@
           <t>meditatie-omslagdoeken-en-accessoires</t>
         </is>
       </c>
-      <c r="F128" s="2" t="inlineStr">
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>alle-meditatiekussens</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>meditatiekussens-rond-biologisch</t>
+        </is>
+      </c>
+      <c r="H128" s="2" t="inlineStr">
         <is>
           <t>cushion -&gt; meditation accessories</t>
         </is>
@@ -3699,7 +4839,17 @@
           <t>meditatie-omslagdoeken-en-accessoires</t>
         </is>
       </c>
-      <c r="F129" s="2" t="inlineStr">
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>biologische-meditatiekussens</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>alle-meditatiekussens</t>
+        </is>
+      </c>
+      <c r="H129" s="2" t="inlineStr">
         <is>
           <t>cushion -&gt; meditation accessories</t>
         </is>
@@ -3725,7 +4875,17 @@
           <t>meditatie-omslagdoeken-en-accessoires</t>
         </is>
       </c>
-      <c r="F130" s="2" t="inlineStr">
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>alle-meditatiekussens</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>meditatiebankjes</t>
+        </is>
+      </c>
+      <c r="H130" s="2" t="inlineStr">
         <is>
           <t>mats -&gt; meditation accessories</t>
         </is>
@@ -3751,7 +4911,17 @@
           <t>massage-hulpmiddelen</t>
         </is>
       </c>
-      <c r="F131" s="2" t="inlineStr">
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>massageolie</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>zorgenstenen-en-knuffelstenen</t>
+        </is>
+      </c>
+      <c r="H131" s="2" t="inlineStr">
         <is>
           <t>meridian balls -&gt; massage tools</t>
         </is>
@@ -3777,7 +4947,17 @@
           <t>ruwe-onbewerkte-mineralen</t>
         </is>
       </c>
-      <c r="F132" s="2" t="inlineStr">
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>edelsteen-bollen</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>edelsteen-piramides-obelisk</t>
+        </is>
+      </c>
+      <c r="H132" s="2" t="inlineStr">
         <is>
           <t>mineral decor &lt;-&gt; raw minerals</t>
         </is>
@@ -3803,7 +4983,7 @@
         </is>
       </c>
       <c r="E133" s="3" t="n"/>
-      <c r="F133" s="3" t="n"/>
+      <c r="H133" s="3" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -3825,7 +5005,17 @@
           <t>wierookhouders-en-accessoires</t>
         </is>
       </c>
-      <c r="F134" s="2" t="inlineStr">
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>alle-wierook</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>masala-en-ayurvedische-wierook</t>
+        </is>
+      </c>
+      <c r="H134" s="2" t="inlineStr">
         <is>
           <t>incense -&gt; needs holder</t>
         </is>
@@ -3851,7 +5041,17 @@
           <t>bad-douche-en-zeep</t>
         </is>
       </c>
-      <c r="F135" s="2" t="inlineStr">
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>lichaamsverzorging-producten</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>biologische-lichaamsverzorging</t>
+        </is>
+      </c>
+      <c r="H135" s="2" t="inlineStr">
         <is>
           <t>Aleppo soap brand -&gt; bath/soap</t>
         </is>
@@ -3877,7 +5077,7 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="F136" s="2" t="inlineStr">
+      <c r="H136" s="2" t="inlineStr">
         <is>
           <t>merch bucket - no logical pair</t>
         </is>
@@ -3903,7 +5103,17 @@
           <t>wierookhouders-en-accessoires</t>
         </is>
       </c>
-      <c r="F137" s="2" t="n"/>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>alle-wierook</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>masala-en-ayurvedische-wierook</t>
+        </is>
+      </c>
+      <c r="H137" s="2" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -3925,7 +5135,17 @@
           <t>postkaarten</t>
         </is>
       </c>
-      <c r="F138" s="2" t="inlineStr">
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>stickers</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>magneten-sleutelhangers-en-gelukspoppetjes</t>
+        </is>
+      </c>
+      <c r="H138" s="2" t="inlineStr">
         <is>
           <t>notebooks -&gt; postcards</t>
         </is>
@@ -3951,7 +5171,17 @@
           <t>alle-etherische-olien</t>
         </is>
       </c>
-      <c r="F139" s="2" t="inlineStr">
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>aroma-diffusers</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>interieur-geurproducten</t>
+        </is>
+      </c>
+      <c r="H139" s="2" t="inlineStr">
         <is>
           <t>diffuser -&gt; needs oils</t>
         </is>
@@ -3977,7 +5207,17 @@
           <t>sieraden-opbergdozen-en-tasjes</t>
         </is>
       </c>
-      <c r="F140" s="2" t="inlineStr">
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>alle-sieraden</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>edelsteen-oorbellen</t>
+        </is>
+      </c>
+      <c r="H140" s="2" t="inlineStr">
         <is>
           <t>jewelry -&gt; storage</t>
         </is>
@@ -4003,7 +5243,17 @@
           <t>lichaamsverzorging-producten</t>
         </is>
       </c>
-      <c r="F141" s="2" t="inlineStr">
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>alle-kaarsen</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>biologische-ontspanningsproducten</t>
+        </is>
+      </c>
+      <c r="H141" s="2" t="inlineStr">
         <is>
           <t>ear/body candles -&gt; body care</t>
         </is>
@@ -4029,7 +5279,17 @@
           <t>mineralen-decoratie-producten</t>
         </is>
       </c>
-      <c r="F142" s="2" t="inlineStr">
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>shungiet-producten</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>feng-shui-kristalproducten</t>
+        </is>
+      </c>
+      <c r="H142" s="2" t="inlineStr">
         <is>
           <t>orgonite -&gt; mineral decor</t>
         </is>
@@ -4055,7 +5315,17 @@
           <t>klein-meubilair-en-decoratie</t>
         </is>
       </c>
-      <c r="F143" s="2" t="inlineStr">
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>banners-wandkleden-en-strandlakens</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>kamerfonteinen</t>
+        </is>
+      </c>
+      <c r="H143" s="2" t="inlineStr">
         <is>
           <t>poufs -&gt; furniture/decor</t>
         </is>
@@ -4081,7 +5351,17 @@
           <t>wierookhouders-en-accessoires</t>
         </is>
       </c>
-      <c r="F144" s="2" t="inlineStr">
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>palo-santo-wierook</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>palo-santo-sieraden</t>
+        </is>
+      </c>
+      <c r="H144" s="2" t="inlineStr">
         <is>
           <t>palo santo -&gt; burning accessories</t>
         </is>
@@ -4107,7 +5387,17 @@
           <t>sieraden-opbergdozen-en-tasjes</t>
         </is>
       </c>
-      <c r="F145" s="2" t="inlineStr">
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>palo-santo-alle-producten</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>alle-sieraden</t>
+        </is>
+      </c>
+      <c r="H145" s="2" t="inlineStr">
         <is>
           <t>jewelry -&gt; storage</t>
         </is>
@@ -4133,7 +5423,17 @@
           <t>wierookhouders-en-accessoires</t>
         </is>
       </c>
-      <c r="F146" s="2" t="n"/>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>palo-santo-alle-producten</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>alle-wierook</t>
+        </is>
+      </c>
+      <c r="H146" s="2" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -4155,7 +5455,17 @@
           <t>lichaamsverzorging-producten</t>
         </is>
       </c>
-      <c r="F147" s="2" t="inlineStr">
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>interieur-geurproducten</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>gezichtsverzorging</t>
+        </is>
+      </c>
+      <c r="H147" s="2" t="inlineStr">
         <is>
           <t>perfume -&gt; body care</t>
         </is>
@@ -4181,7 +5491,17 @@
           <t>pendels-van-mineralen-hout-en-rudraksha</t>
         </is>
       </c>
-      <c r="F148" s="2" t="inlineStr">
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>pendels-voor-professionals</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>biotensors-en-wichelroedes</t>
+        </is>
+      </c>
+      <c r="H148" s="2" t="inlineStr">
         <is>
           <t>accessories -&gt; pendulums</t>
         </is>
@@ -4207,7 +5527,17 @@
           <t>pendel-accessoires</t>
         </is>
       </c>
-      <c r="F149" s="2" t="inlineStr">
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>pendels-voor-professionals</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>biotensors-en-wichelroedes</t>
+        </is>
+      </c>
+      <c r="H149" s="2" t="inlineStr">
         <is>
           <t>pendulums -&gt; pendulum accessories</t>
         </is>
@@ -4233,7 +5563,17 @@
           <t>pendel-accessoires</t>
         </is>
       </c>
-      <c r="F150" s="2" t="inlineStr">
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>pendels-van-mineralen-hout-en-rudraksha</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>biotensors-en-wichelroedes</t>
+        </is>
+      </c>
+      <c r="H150" s="2" t="inlineStr">
         <is>
           <t>pro pendulums -&gt; pendulum accessories</t>
         </is>
@@ -4259,7 +5599,17 @@
           <t>notitieboeken-en-meer</t>
         </is>
       </c>
-      <c r="F151" s="2" t="inlineStr">
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>stickers</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>magneten-sleutelhangers-en-gelukspoppetjes</t>
+        </is>
+      </c>
+      <c r="H151" s="2" t="inlineStr">
         <is>
           <t>postcards -&gt; notebooks</t>
         </is>
@@ -4285,7 +5635,7 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="F152" s="2" t="inlineStr">
+      <c r="H152" s="2" t="inlineStr">
         <is>
           <t>don't associate, remove from final file</t>
         </is>
@@ -4311,7 +5661,17 @@
           <t>stickers</t>
         </is>
       </c>
-      <c r="F153" s="2" t="inlineStr">
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>illumination-mandala-stickers</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>postkaarten</t>
+        </is>
+      </c>
+      <c r="H153" s="2" t="inlineStr">
         <is>
           <t>window stickers -&gt; stickers</t>
         </is>
@@ -4337,7 +5697,17 @@
           <t>sieraden-opbergdozen-en-tasjes</t>
         </is>
       </c>
-      <c r="F154" s="2" t="inlineStr">
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>alle-sieraden</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>edelsteen-ringen</t>
+        </is>
+      </c>
+      <c r="H154" s="2" t="inlineStr">
         <is>
           <t>jewelry -&gt; storage</t>
         </is>
@@ -4363,7 +5733,17 @@
           <t>witte-salie-en-smudges</t>
         </is>
       </c>
-      <c r="F155" s="2" t="inlineStr">
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>wicca-en-tarot</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>kathas-altaar-en-deurkleden</t>
+        </is>
+      </c>
+      <c r="H155" s="2" t="inlineStr">
         <is>
           <t>ritual objects -&gt; sage/smudge</t>
         </is>
@@ -4389,7 +5769,17 @@
           <t>ruwe-onbewerkte-mineralen</t>
         </is>
       </c>
-      <c r="F156" s="2" t="inlineStr">
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>trommelstenen</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>mineralen-decoratie-producten</t>
+        </is>
+      </c>
+      <c r="H156" s="2" t="inlineStr">
         <is>
           <t>power boxes -&gt; raw minerals</t>
         </is>
@@ -4415,7 +5805,17 @@
           <t>mineralen-decoratie-producten</t>
         </is>
       </c>
-      <c r="F157" s="2" t="inlineStr">
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>trommelstenen</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>ruwe-edelstenen-power-boxen</t>
+        </is>
+      </c>
+      <c r="H157" s="2" t="inlineStr">
         <is>
           <t>raw minerals &lt;-&gt; mineral decor</t>
         </is>
@@ -4441,7 +5841,17 @@
           <t>wierookhouders-en-accessoires</t>
         </is>
       </c>
-      <c r="F158" s="2" t="n"/>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>alle-wierook</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>witte-salie-en-smudges</t>
+        </is>
+      </c>
+      <c r="H158" s="2" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -4463,7 +5873,17 @@
           <t>lichaamsverzorging-producten</t>
         </is>
       </c>
-      <c r="F159" s="2" t="inlineStr">
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>bad-douche-en-zeep</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>gezichtsverzorging</t>
+        </is>
+      </c>
+      <c r="H159" s="2" t="inlineStr">
         <is>
           <t>cosmetics brand -&gt; body care</t>
         </is>
@@ -4489,7 +5909,17 @@
           <t>edelsteen-en-seleniet-lampen</t>
         </is>
       </c>
-      <c r="F160" s="2" t="inlineStr">
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>mineralen-decoratie-producten</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>zoutlampen-en-meer</t>
+        </is>
+      </c>
+      <c r="H160" s="2" t="inlineStr">
         <is>
           <t>selenite -&gt; selenite lamps</t>
         </is>
@@ -4515,7 +5945,7 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="F161" s="2" t="inlineStr">
+      <c r="H161" s="2" t="inlineStr">
         <is>
           <t>merch bucket - no logical pair</t>
         </is>
@@ -4541,7 +5971,17 @@
           <t>alle-kaarsen</t>
         </is>
       </c>
-      <c r="F162" s="2" t="inlineStr">
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>geurkaarsen</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>waxinelichtjes</t>
+        </is>
+      </c>
+      <c r="H162" s="2" t="inlineStr">
         <is>
           <t>holders -&gt; need candles</t>
         </is>
@@ -4567,7 +6007,17 @@
           <t>mineralen-decoratie-producten</t>
         </is>
       </c>
-      <c r="F163" s="2" t="inlineStr">
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>orgoniet-producten</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>ruwe-onbewerkte-mineralen</t>
+        </is>
+      </c>
+      <c r="H163" s="2" t="inlineStr">
         <is>
           <t>shungite -&gt; mineral decor</t>
         </is>
@@ -4593,7 +6043,7 @@
         </is>
       </c>
       <c r="E164" s="3" t="n"/>
-      <c r="F164" s="3" t="n"/>
+      <c r="H164" s="3" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -4615,7 +6065,17 @@
           <t>alle-sieraden</t>
         </is>
       </c>
-      <c r="F165" s="2" t="inlineStr">
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>sieraden-opbergdozen-en-tasjes</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>edelsteen-armbanden</t>
+        </is>
+      </c>
+      <c r="H165" s="2" t="inlineStr">
         <is>
           <t>jewelry accessories -&gt; all jewelry</t>
         </is>
@@ -4641,7 +6101,17 @@
           <t>sieraden-opbergdozen-en-tasjes</t>
         </is>
       </c>
-      <c r="F166" s="2" t="inlineStr">
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>bloem-des-levens-producten</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>alle-sieraden</t>
+        </is>
+      </c>
+      <c r="H166" s="2" t="inlineStr">
         <is>
           <t>jewelry -&gt; storage</t>
         </is>
@@ -4667,7 +6137,17 @@
           <t>sieraden-opbergdozen-en-tasjes</t>
         </is>
       </c>
-      <c r="F167" s="2" t="inlineStr">
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>alle-sieraden</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>oorbellen</t>
+        </is>
+      </c>
+      <c r="H167" s="2" t="inlineStr">
         <is>
           <t>jewelry -&gt; storage</t>
         </is>
@@ -4693,7 +6173,17 @@
           <t>sieraden-opbergdozen-en-tasjes</t>
         </is>
       </c>
-      <c r="F168" s="2" t="inlineStr">
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>chakra-producten</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>alle-sieraden</t>
+        </is>
+      </c>
+      <c r="H168" s="2" t="inlineStr">
         <is>
           <t>jewelry -&gt; storage</t>
         </is>
@@ -4719,7 +6209,17 @@
           <t>sieraden-opbergdozen-en-tasjes</t>
         </is>
       </c>
-      <c r="F169" s="2" t="inlineStr">
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>engel-producten</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>alle-sieraden</t>
+        </is>
+      </c>
+      <c r="H169" s="2" t="inlineStr">
         <is>
           <t>jewelry -&gt; storage</t>
         </is>
@@ -4745,7 +6245,17 @@
           <t>alle-sieraden</t>
         </is>
       </c>
-      <c r="F170" s="2" t="inlineStr">
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>verpakkingen-potjes-dozen-tasjes</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>tassen-en-tasjes</t>
+        </is>
+      </c>
+      <c r="H170" s="2" t="inlineStr">
         <is>
           <t>storage -&gt; all jewelry</t>
         </is>
@@ -4771,7 +6281,17 @@
           <t>tassen-en-tasjes</t>
         </is>
       </c>
-      <c r="F171" s="2" t="inlineStr">
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>meditatie-omslagdoeken-en-accessoires</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>yoga-omslagdoeken</t>
+        </is>
+      </c>
+      <c r="H171" s="2" t="inlineStr">
         <is>
           <t>scarves -&gt; bags</t>
         </is>
@@ -4797,7 +6317,17 @@
           <t>olieverdampers-en-geurstenen</t>
         </is>
       </c>
-      <c r="F172" s="2" t="inlineStr">
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>alle-etherische-olien</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>song-of-india-r-expo-wierook</t>
+        </is>
+      </c>
+      <c r="H172" s="2" t="inlineStr">
         <is>
           <t>oils -&gt; diffuser</t>
         </is>
@@ -4823,7 +6353,17 @@
           <t>wierookhouders-en-accessoires</t>
         </is>
       </c>
-      <c r="F173" s="2" t="inlineStr">
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>song-of-india-r-expo-wierook</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>song-of-india-essentiele-olien</t>
+        </is>
+      </c>
+      <c r="H173" s="2" t="inlineStr">
         <is>
           <t>brand mostly incense -&gt; holders</t>
         </is>
@@ -4849,7 +6389,17 @@
           <t>wierookhouders-en-accessoires</t>
         </is>
       </c>
-      <c r="F174" s="2" t="n"/>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>alle-wierook</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>song-of-india-essentiele-olien</t>
+        </is>
+      </c>
+      <c r="H174" s="2" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
@@ -4871,7 +6421,17 @@
           <t>accessoires-metalen-klankschalen</t>
         </is>
       </c>
-      <c r="F175" s="2" t="inlineStr">
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>alle-metalen-klankschalen</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>gongs-gongtassen-en-gongstandaards</t>
+        </is>
+      </c>
+      <c r="H175" s="2" t="inlineStr">
         <is>
           <t>sound healing -&gt; bowl accessories</t>
         </is>
@@ -4897,7 +6457,7 @@
         </is>
       </c>
       <c r="E176" s="3" t="n"/>
-      <c r="F176" s="3" t="n"/>
+      <c r="H176" s="3" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="3" t="inlineStr">
@@ -4919,7 +6479,7 @@
         </is>
       </c>
       <c r="E177" s="3" t="n"/>
-      <c r="F177" s="3" t="n"/>
+      <c r="H177" s="3" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="3" t="inlineStr">
@@ -4941,7 +6501,7 @@
         </is>
       </c>
       <c r="E178" s="3" t="n"/>
-      <c r="F178" s="3" t="n"/>
+      <c r="H178" s="3" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
@@ -4963,7 +6523,17 @@
           <t>sound-healing-instrumenten</t>
         </is>
       </c>
-      <c r="F179" s="2" t="inlineStr">
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>klankbuizen-en-klankstaven</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>alle-metalen-klankschalen</t>
+        </is>
+      </c>
+      <c r="H179" s="2" t="inlineStr">
         <is>
           <t>tuning forks -&gt; sound healing range</t>
         </is>
@@ -4989,7 +6559,17 @@
           <t>raamstickers</t>
         </is>
       </c>
-      <c r="F180" s="2" t="inlineStr">
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>illumination-mandala-stickers</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>postkaarten</t>
+        </is>
+      </c>
+      <c r="H180" s="2" t="inlineStr">
         <is>
           <t>stickers -&gt; window stickers</t>
         </is>
@@ -5015,7 +6595,17 @@
           <t>lichaamsverzorging-producten</t>
         </is>
       </c>
-      <c r="F181" s="2" t="inlineStr">
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>gezichtsverzorging</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>bad-douche-en-zeep</t>
+        </is>
+      </c>
+      <c r="H181" s="2" t="inlineStr">
         <is>
           <t>sulfur care -&gt; body care</t>
         </is>
@@ -5041,7 +6631,17 @@
           <t>sjaals-en-pashminas</t>
         </is>
       </c>
-      <c r="F182" s="2" t="inlineStr">
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>sieraden-opbergdozen-en-tasjes</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>malas-en-mala-tasjes</t>
+        </is>
+      </c>
+      <c r="H182" s="2" t="inlineStr">
         <is>
           <t>bags -&gt; scarves</t>
         </is>
@@ -5067,7 +6667,7 @@
         </is>
       </c>
       <c r="E183" s="3" t="n"/>
-      <c r="F183" s="3" t="n"/>
+      <c r="H183" s="3" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="3" t="inlineStr">
@@ -5089,7 +6689,7 @@
         </is>
       </c>
       <c r="E184" s="3" t="n"/>
-      <c r="F184" s="3" t="n"/>
+      <c r="H184" s="3" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
@@ -5111,7 +6711,17 @@
           <t>thee-alle-producten</t>
         </is>
       </c>
-      <c r="F185" s="2" t="inlineStr">
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>biologische-thee</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>thee-shoti-maa-biologisch</t>
+        </is>
+      </c>
+      <c r="H185" s="2" t="inlineStr">
         <is>
           <t>tea accessories -&gt; tea</t>
         </is>
@@ -5137,7 +6747,17 @@
           <t>thee-accessoires</t>
         </is>
       </c>
-      <c r="F186" s="2" t="inlineStr">
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>biologische-thee</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>thee-shoti-maa-biologisch</t>
+        </is>
+      </c>
+      <c r="H186" s="2" t="inlineStr">
         <is>
           <t>tea -&gt; tea accessories</t>
         </is>
@@ -5163,7 +6783,17 @@
           <t>thee-accessoires</t>
         </is>
       </c>
-      <c r="F187" s="2" t="inlineStr">
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>thee-alle-producten</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>biologische-thee</t>
+        </is>
+      </c>
+      <c r="H187" s="2" t="inlineStr">
         <is>
           <t>tea -&gt; tea accessories</t>
         </is>
@@ -5189,7 +6819,17 @@
           <t>thee-accessoires</t>
         </is>
       </c>
-      <c r="F188" s="2" t="inlineStr">
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>thee-alle-producten</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>biologische-thee</t>
+        </is>
+      </c>
+      <c r="H188" s="2" t="inlineStr">
         <is>
           <t>tea -&gt; tea accessories</t>
         </is>
@@ -5215,7 +6855,17 @@
           <t>thee-accessoires</t>
         </is>
       </c>
-      <c r="F189" s="2" t="inlineStr">
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>thee-alle-producten</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>biologische-thee</t>
+        </is>
+      </c>
+      <c r="H189" s="2" t="inlineStr">
         <is>
           <t>tea -&gt; tea accessories</t>
         </is>
@@ -5241,7 +6891,17 @@
           <t>tibetaanse-producten</t>
         </is>
       </c>
-      <c r="F190" s="2" t="inlineStr">
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>banners-wandkleden-en-strandlakens</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>tibetaanse-wierook</t>
+        </is>
+      </c>
+      <c r="H190" s="2" t="inlineStr">
         <is>
           <t>prayer flags -&gt; Tibetan range</t>
         </is>
@@ -5267,7 +6927,17 @@
           <t>tibetaanse-gebedsvlaggen</t>
         </is>
       </c>
-      <c r="F191" s="2" t="inlineStr">
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>tibetaanse-wierook</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>klein-meubilair-en-decoratie</t>
+        </is>
+      </c>
+      <c r="H191" s="2" t="inlineStr">
         <is>
           <t>Tibetan range -&gt; prayer flags</t>
         </is>
@@ -5293,7 +6963,17 @@
           <t>wierookhouders-en-accessoires</t>
         </is>
       </c>
-      <c r="F192" s="2" t="n"/>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>alle-wierook</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>tibetaanse-producten</t>
+        </is>
+      </c>
+      <c r="H192" s="2" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
@@ -5315,7 +6995,17 @@
           <t>zorgenstenen-en-knuffelstenen</t>
         </is>
       </c>
-      <c r="F193" s="2" t="inlineStr">
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>trommelstenen-mini-chips</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>ruwe-onbewerkte-mineralen</t>
+        </is>
+      </c>
+      <c r="H193" s="2" t="inlineStr">
         <is>
           <t>tumbled stones -&gt; worry/cuddle stones</t>
         </is>
@@ -5341,7 +7031,17 @@
           <t>trommelstenen</t>
         </is>
       </c>
-      <c r="F194" s="2" t="inlineStr">
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>zorgenstenen-en-knuffelstenen</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>ruwe-onbewerkte-mineralen</t>
+        </is>
+      </c>
+      <c r="H194" s="2" t="inlineStr">
         <is>
           <t>mini chips -&gt; tumbled stones</t>
         </is>
@@ -5367,7 +7067,17 @@
           <t>klein-meubilair-en-decoratie</t>
         </is>
       </c>
-      <c r="F195" s="2" t="inlineStr">
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>windorgels-en-windbellen</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>kamerfonteinen</t>
+        </is>
+      </c>
+      <c r="H195" s="2" t="inlineStr">
         <is>
           <t>garden -&gt; decor</t>
         </is>
@@ -5393,7 +7103,7 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="F196" s="2" t="inlineStr">
+      <c r="H196" s="2" t="inlineStr">
         <is>
           <t>merch bucket - no logical pair</t>
         </is>
@@ -5419,7 +7129,17 @@
           <t>sieraden-opbergdozen-en-tasjes</t>
         </is>
       </c>
-      <c r="F197" s="2" t="inlineStr">
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>tassen-en-tasjes</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>notitieboeken-en-meer</t>
+        </is>
+      </c>
+      <c r="H197" s="2" t="inlineStr">
         <is>
           <t>packaging -&gt; jewelry storage</t>
         </is>
@@ -5445,7 +7165,17 @@
           <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
-      <c r="F198" s="2" t="inlineStr">
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>alle-kaarsen</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>honderd-uur-kaarsen</t>
+        </is>
+      </c>
+      <c r="H198" s="2" t="inlineStr">
         <is>
           <t>candles -&gt; holders/lights</t>
         </is>
@@ -5471,7 +7201,17 @@
           <t>meditatie-drinkflessen</t>
         </is>
       </c>
-      <c r="F199" s="2" t="inlineStr">
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>watervitalisering-vitajuwel</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>watervitalisering-natures-design</t>
+        </is>
+      </c>
+      <c r="H199" s="2" t="inlineStr">
         <is>
           <t>water vitalization -&gt; gemstone bottles</t>
         </is>
@@ -5497,7 +7237,17 @@
           <t>watervitalisering-alle-producten</t>
         </is>
       </c>
-      <c r="F200" s="2" t="inlineStr">
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>watervitalisering-mineraalstaven</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>meditatie-drinkflessen</t>
+        </is>
+      </c>
+      <c r="H200" s="2" t="inlineStr">
         <is>
           <t>-&gt; full water range</t>
         </is>
@@ -5523,7 +7273,17 @@
           <t>watervitalisering-alle-producten</t>
         </is>
       </c>
-      <c r="F201" s="2" t="inlineStr">
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>watervitalisering-edelsteenstaven</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>meditatie-drinkflessen</t>
+        </is>
+      </c>
+      <c r="H201" s="2" t="inlineStr">
         <is>
           <t>-&gt; full water range</t>
         </is>
@@ -5549,7 +7309,17 @@
           <t>watervitalisering-alle-producten</t>
         </is>
       </c>
-      <c r="F202" s="2" t="inlineStr">
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>meditatie-drinkflessen</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>watervitalisering-vitajuwel</t>
+        </is>
+      </c>
+      <c r="H202" s="2" t="inlineStr">
         <is>
           <t>-&gt; full water range</t>
         </is>
@@ -5575,7 +7345,17 @@
           <t>watervitalisering-alle-producten</t>
         </is>
       </c>
-      <c r="F203" s="2" t="inlineStr">
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>meditatie-drinkflessen</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>watervitalisering-natures-design</t>
+        </is>
+      </c>
+      <c r="H203" s="2" t="inlineStr">
         <is>
           <t>-&gt; full water range</t>
         </is>
@@ -5601,7 +7381,17 @@
           <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
-      <c r="F204" s="2" t="inlineStr">
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>zoutkristal-kaarshouders</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>alle-kaarsen</t>
+        </is>
+      </c>
+      <c r="H204" s="2" t="inlineStr">
         <is>
           <t>tealights -&gt; holders/lights</t>
         </is>
@@ -5627,7 +7417,17 @@
           <t>rituele-voorwerpen</t>
         </is>
       </c>
-      <c r="F205" s="2" t="inlineStr">
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>witte-salie-en-smudges</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>chakra-en-wicca-mineraalsets</t>
+        </is>
+      </c>
+      <c r="H205" s="2" t="inlineStr">
         <is>
           <t>wicca/tarot -&gt; ritual objects</t>
         </is>
@@ -5653,7 +7453,7 @@
         </is>
       </c>
       <c r="E206" s="3" t="n"/>
-      <c r="F206" s="3" t="n"/>
+      <c r="H206" s="3" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
@@ -5675,7 +7475,17 @@
           <t>houtskool-en-houtkoolbranders</t>
         </is>
       </c>
-      <c r="F207" s="2" t="inlineStr">
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>alle-wierook</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>witte-salie-en-smudges</t>
+        </is>
+      </c>
+      <c r="H207" s="2" t="inlineStr">
         <is>
           <t>resins/herbs burn on charcoal</t>
         </is>
@@ -5701,7 +7511,17 @@
           <t>alle-wierook</t>
         </is>
       </c>
-      <c r="F208" s="2" t="inlineStr">
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>wierookharsen-en-wierookkruiden</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>houtskool-en-houtkoolbranders</t>
+        </is>
+      </c>
+      <c r="H208" s="2" t="inlineStr">
         <is>
           <t>holders/accessories -&gt; all incense</t>
         </is>
@@ -5727,7 +7547,17 @@
           <t>wierookhouders-en-accessoires</t>
         </is>
       </c>
-      <c r="F209" s="2" t="n"/>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>alle-wierook</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>backflow-branders-kegels</t>
+        </is>
+      </c>
+      <c r="H209" s="2" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
@@ -5749,7 +7579,17 @@
           <t>feng-shui-producten</t>
         </is>
       </c>
-      <c r="F210" s="2" t="inlineStr">
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>tuin-en-buiten</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>klein-meubilair-en-decoratie</t>
+        </is>
+      </c>
+      <c r="H210" s="2" t="inlineStr">
         <is>
           <t>wind chimes -&gt; feng shui</t>
         </is>
@@ -5775,7 +7615,17 @@
           <t>wierookhouders-en-accessoires</t>
         </is>
       </c>
-      <c r="F211" s="2" t="inlineStr">
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>wierookharsen-en-wierookkruiden</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>rituele-voorwerpen</t>
+        </is>
+      </c>
+      <c r="H211" s="2" t="inlineStr">
         <is>
           <t>smudge -&gt; burning accessories</t>
         </is>
@@ -5801,7 +7651,7 @@
         </is>
       </c>
       <c r="E212" s="3" t="n"/>
-      <c r="F212" s="3" t="n"/>
+      <c r="H212" s="3" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
@@ -5823,7 +7673,17 @@
           <t>yogamatten-en-handdoeken</t>
         </is>
       </c>
-      <c r="F213" s="2" t="inlineStr">
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>yogariemen-en-yogawiel</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>yoga-welzijn</t>
+        </is>
+      </c>
+      <c r="H213" s="2" t="inlineStr">
         <is>
           <t>yoga prop -&gt; mats</t>
         </is>
@@ -5849,7 +7709,17 @@
           <t>yogamatten-en-handdoeken</t>
         </is>
       </c>
-      <c r="F214" s="2" t="inlineStr">
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>yoga-welzijn</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>sjaals-en-pashminas</t>
+        </is>
+      </c>
+      <c r="H214" s="2" t="inlineStr">
         <is>
           <t>yoga textile -&gt; mats</t>
         </is>
@@ -5875,7 +7745,17 @@
           <t>yogamatten-en-handdoeken</t>
         </is>
       </c>
-      <c r="F215" s="2" t="inlineStr">
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>yogariemen-en-yogawiel</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>yoga-bolsters</t>
+        </is>
+      </c>
+      <c r="H215" s="2" t="inlineStr">
         <is>
           <t>yoga prop -&gt; mats</t>
         </is>
@@ -5901,7 +7781,17 @@
           <t>yogamatten-en-handdoeken</t>
         </is>
       </c>
-      <c r="F216" s="2" t="inlineStr">
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>biologische-yogaproducten</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>yoga-wierook</t>
+        </is>
+      </c>
+      <c r="H216" s="2" t="inlineStr">
         <is>
           <t>yoga wellness -&gt; mats</t>
         </is>
@@ -5927,7 +7817,17 @@
           <t>wierookhouders-en-accessoires</t>
         </is>
       </c>
-      <c r="F217" s="2" t="n"/>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>alle-wierook</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>yoga-welzijn</t>
+        </is>
+      </c>
+      <c r="H217" s="2" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
@@ -5949,7 +7849,17 @@
           <t>yogariemen-en-yogawiel</t>
         </is>
       </c>
-      <c r="F218" s="2" t="inlineStr">
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>yoga-props-kurk</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>yogamatten-reiniger-biologisch</t>
+        </is>
+      </c>
+      <c r="H218" s="2" t="inlineStr">
         <is>
           <t>mats -&gt; straps/wheel</t>
         </is>
@@ -5975,7 +7885,17 @@
           <t>yogamatten-en-handdoeken</t>
         </is>
       </c>
-      <c r="F219" s="2" t="inlineStr">
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>biologische-yogaproducten</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>yoga-welzijn</t>
+        </is>
+      </c>
+      <c r="H219" s="2" t="inlineStr">
         <is>
           <t>mat cleaner -&gt; mats</t>
         </is>
@@ -6001,7 +7921,17 @@
           <t>yogamatten-en-handdoeken</t>
         </is>
       </c>
-      <c r="F220" s="2" t="inlineStr">
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>yoga-props-kurk</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>yoga-bolsters</t>
+        </is>
+      </c>
+      <c r="H220" s="2" t="inlineStr">
         <is>
           <t>straps/wheel -&gt; mats</t>
         </is>
@@ -6027,7 +7957,17 @@
           <t>wierookhouders-en-accessoires</t>
         </is>
       </c>
-      <c r="F221" s="2" t="inlineStr">
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>klein-meubilair-en-decoratie</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>backflow-branders-kegels</t>
+        </is>
+      </c>
+      <c r="H221" s="2" t="inlineStr">
         <is>
           <t>soapstone items incl. incense holders</t>
         </is>
@@ -6053,7 +7993,17 @@
           <t>trommelstenen</t>
         </is>
       </c>
-      <c r="F222" s="2" t="inlineStr">
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>trommelstenen-mini-chips</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>ruwe-onbewerkte-mineralen</t>
+        </is>
+      </c>
+      <c r="H222" s="2" t="inlineStr">
         <is>
           <t>worry stones -&gt; tumbled stones</t>
         </is>
@@ -6079,7 +8029,17 @@
           <t>waxinelichtjes</t>
         </is>
       </c>
-      <c r="F223" s="2" t="inlineStr">
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>sfeerlichten-en-lantaarns</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>zoutlampen-en-meer</t>
+        </is>
+      </c>
+      <c r="H223" s="2" t="inlineStr">
         <is>
           <t>salt candle holders -&gt; tealights</t>
         </is>
@@ -6105,7 +8065,17 @@
           <t>klein-meubilair-en-decoratie</t>
         </is>
       </c>
-      <c r="F224" s="2" t="inlineStr">
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>zoutkristal-kaarshouders</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>seleniet-producten</t>
+        </is>
+      </c>
+      <c r="H224" s="2" t="inlineStr">
         <is>
           <t>salt lamps -&gt; decor</t>
         </is>

</xml_diff>

<commit_message>
Rework match_2/match_3 to complementary companions
Replace same-category 'broader range' substitutes with genuine
cross-sell companions (the basket a buyer also needs): e.g. singing
bowl -> cushion + incense; gemstones -> selenite + sage + pouch;
jewelry -> storage + findings + gift packaging; statue -> incense +
altar cloth. match_1 preserved; all targets published, in-stock,
distinct.
</commit_message>
<xml_diff>
--- a/phoenix_collections_pairing_map_FILLED.xlsx
+++ b/phoenix_collections_pairing_map_FILLED.xlsx
@@ -521,7 +521,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>alle-wierook</t>
+          <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -553,12 +553,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>sound-healing-instrumenten</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>accessoires-metalen-klankschalen</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="H3" s="2" t="n"/>
@@ -585,12 +585,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>sound-healing-instrumenten</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>accessoires-kristallen-klankschalen</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="H4" s="2" t="n"/>
@@ -617,12 +617,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>alle-wierook</t>
+          <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>masala-en-ayurvedische-wierook</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="H5" s="2" t="n"/>
@@ -649,12 +649,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>boeddha-beelden</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>hindoe-beelden</t>
+          <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
       <c r="H6" s="2" t="n"/>
@@ -681,12 +681,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>biologische-etherische-olie</t>
+          <t>aroma-diffusers</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>aroma-diffusers</t>
+          <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
       <c r="H7" s="2" t="n"/>
@@ -713,12 +713,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>geurkaarsen</t>
+          <t>zoutkristal-kaarshouders</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>zoutkristal-kaarshouders</t>
+          <t>klein-meubilair-en-decoratie</t>
         </is>
       </c>
       <c r="H8" s="2" t="n"/>
@@ -745,12 +745,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
+          <t>alle-meditatiekussens</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
           <t>sound-healing-instrumenten</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>alle-metalen-klankschalen</t>
         </is>
       </c>
       <c r="H9" s="2" t="n"/>
@@ -777,12 +777,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>meditatiematten-en-meditatiesets</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>meditatiebankjes</t>
+          <t>alle-metalen-klankschalen</t>
         </is>
       </c>
       <c r="H10" s="2" t="n"/>
@@ -809,12 +809,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
+          <t>alle-meditatiekussens</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
           <t>sound-healing-instrumenten</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>alle-kristallen-klankschalen</t>
         </is>
       </c>
       <c r="H11" s="2" t="n"/>
@@ -841,12 +841,12 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>edelsteen-armbanden</t>
+          <t>sieraden-accessoires</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>edelsteen-hangers-gepolijst</t>
+          <t>verpakkingen-potjes-dozen-tasjes</t>
         </is>
       </c>
       <c r="H12" s="2" t="n"/>
@@ -873,12 +873,12 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>houtskool-en-houtkoolbranders</t>
+          <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>wierookharsen-en-wierookkruiden</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="H13" s="2" t="n"/>
@@ -905,12 +905,12 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>alle-sieraden</t>
+          <t>sieraden-accessoires</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>edelsteen-armbanden</t>
+          <t>verpakkingen-potjes-dozen-tasjes</t>
         </is>
       </c>
       <c r="H14" s="2" t="n"/>
@@ -937,12 +937,12 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>alle-sieraden</t>
+          <t>sieraden-accessoires</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>hangers-metaal</t>
+          <t>verpakkingen-potjes-dozen-tasjes</t>
         </is>
       </c>
       <c r="H15" s="2" t="n"/>
@@ -969,12 +969,12 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>olieverdampers-en-geurstenen</t>
+          <t>biologische-etherische-olie</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>interieur-geurproducten</t>
+          <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
       <c r="H16" s="2" t="n"/>
@@ -1001,12 +1001,12 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>aromafume-geurproducten</t>
+          <t>wierookhouders-en-accessoires</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>aromafume-wierookblokjes-non-toxic</t>
+          <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
       <c r="H17" s="4" t="n"/>
@@ -1033,12 +1033,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>aromafume-alle-producten</t>
+          <t>wierookhouders-en-accessoires</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>interieur-geurproducten</t>
+          <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
       <c r="H18" s="2" t="n"/>
@@ -1065,12 +1065,12 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>aromafume-alle-producten</t>
+          <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>alle-wierook</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>lichaamsverzorging-producten</t>
+          <t>biologische-thee</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>lichaamsverzorging-producten</t>
+          <t>biologische-thee</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1173,12 +1173,12 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>wierookkegels</t>
+          <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>alle-wierook</t>
+          <t>klein-meubilair-en-decoratie</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1209,12 +1209,12 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>biologische-lichaamsverzorging</t>
+          <t>haarverzorging</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>haarverzorging</t>
+          <t>gezichtsverzorging</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -1250,7 +1250,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>tibetaanse-gebedsvlaggen</t>
+          <t>alle-beelden</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1303,12 +1303,12 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>edelsteen-hangers-gepolijst</t>
+          <t>witte-salie-en-smudges</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>alle-sieraden</t>
+          <t>sieraden-accessoires</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -1365,12 +1365,12 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>alle-kaarsen</t>
+          <t>zoutkristal-kaarshouders</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>dinerkaarsen-en-stompkaarsen</t>
+          <t>klein-meubilair-en-decoratie</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1401,12 +1401,12 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>alle-etherische-olien</t>
+          <t>aroma-diffusers</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>aroma-diffusers</t>
+          <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -1442,7 +1442,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>biologische-ontspanningsproducten</t>
+          <t>gezichtsverzorging</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -1473,12 +1473,12 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>alle-meditatiekussens</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>meditatiekussens-rond-biologisch</t>
+          <t>alle-metalen-klankschalen</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -1514,7 +1514,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>bach-bloesem-producten</t>
+          <t>massageolie</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -1567,12 +1567,12 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>thee-alle-producten</t>
+          <t>biologische-ontspanningsproducten</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>thee-shoti-maa-biologisch</t>
+          <t>geurkaarsen</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -1603,12 +1603,12 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
+          <t>yogariemen-en-yogawiel</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
           <t>yoga-welzijn</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>biologische-meditatiekussens</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -1711,12 +1711,12 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>alle-beelden</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>hindoe-beelden</t>
+          <t>kathas-altaar-en-deurkleden</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -1773,12 +1773,12 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
+          <t>wicca-en-tarot</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
           <t>trommelstenen</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>wicca-en-tarot</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -1845,12 +1845,12 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>alle-kaarsen</t>
+          <t>zoutkristal-kaarshouders</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>zoutkristal-kaarshouders</t>
+          <t>klein-meubilair-en-decoratie</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -1881,12 +1881,12 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>alle-sieraden</t>
+          <t>sieraden-accessoires</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>armbanden-edelsteen-aa</t>
+          <t>verpakkingen-potjes-dozen-tasjes</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -1917,12 +1917,12 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>edelsteen-piramides-obelisk</t>
+          <t>klein-meubilair-en-decoratie</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>ruwe-onbewerkte-mineralen</t>
+          <t>seleniet-producten</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -1958,7 +1958,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>mineralen-decoratie-producten</t>
+          <t>klein-meubilair-en-decoratie</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>engelen-beelden</t>
+          <t>engelenkaarsen</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -2025,12 +2025,12 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>hangers-edelsteen-geboord</t>
+          <t>sieraden-accessoires</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>alle-sieraden</t>
+          <t>verpakkingen-potjes-dozen-tasjes</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -2061,12 +2061,12 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>edelsteen-hangers-gepolijst</t>
+          <t>sieraden-accessoires</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>alle-sieraden</t>
+          <t>verpakkingen-potjes-dozen-tasjes</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -2097,12 +2097,12 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>alle-sieraden</t>
+          <t>sieraden-accessoires</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>oorbellen</t>
+          <t>verpakkingen-potjes-dozen-tasjes</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>edelsteen-bollen</t>
+          <t>klein-meubilair-en-decoratie</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2169,12 +2169,12 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>alle-sieraden</t>
+          <t>sieraden-accessoires</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>ringen</t>
+          <t>verpakkingen-potjes-dozen-tasjes</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -2241,12 +2241,12 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>sieraden-engelen</t>
+          <t>engelenkaarsen</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>edelsteen-engelen</t>
+          <t>aartsengelen-wierook</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -2277,12 +2277,12 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
+          <t>engelenkaarsen</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
           <t>engel-producten</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>alle-beelden</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -2313,12 +2313,12 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>alle-kaarsen</t>
+          <t>engel-producten</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>engel-producten</t>
+          <t>zoutkristal-kaarshouders</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -2390,7 +2390,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>mineralen-decoratie-producten</t>
+          <t>windorgels-en-windbellen</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -2421,7 +2421,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>alle-etherische-olien</t>
+          <t>aroma-diffusers</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -2457,12 +2457,12 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>alle-wierook</t>
+          <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>fiore-doriente-essentiele-olien</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="H59" s="2" t="n"/>
@@ -2489,7 +2489,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>alle-kaarsen</t>
+          <t>zoutkristal-kaarshouders</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -2552,7 +2552,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>biologische-lichaamsverzorging</t>
+          <t>haarverzorging</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -2605,12 +2605,12 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>alle-metalen-klankschalen</t>
+          <t>accessoires-metalen-klankschalen</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>stemvorken</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -2677,12 +2677,12 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>edelsteen-hangers-gepolijst</t>
+          <t>sieraden-accessoires</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>alle-sieraden</t>
+          <t>verpakkingen-potjes-dozen-tasjes</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
@@ -2713,12 +2713,12 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>edelsteen-hangers-gepolijst</t>
+          <t>sieraden-accessoires</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>alle-sieraden</t>
+          <t>verpakkingen-potjes-dozen-tasjes</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
@@ -2749,12 +2749,12 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>hangers-overig</t>
+          <t>sieraden-accessoires</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>alle-sieraden</t>
+          <t>verpakkingen-potjes-dozen-tasjes</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
@@ -2785,12 +2785,12 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>hangers-metaal</t>
+          <t>sieraden-accessoires</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>alle-sieraden</t>
+          <t>verpakkingen-potjes-dozen-tasjes</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
@@ -2893,12 +2893,12 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>alle-beelden</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>boeddha-beelden</t>
+          <t>kathas-altaar-en-deurkleden</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
@@ -3009,12 +3009,12 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>alle-kaarsen</t>
+          <t>zoutkristal-kaarshouders</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>votiefkaarsen</t>
+          <t>klein-meubilair-en-decoratie</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
@@ -3045,7 +3045,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>alle-wierook</t>
+          <t>wierookhouders-en-accessoires</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -3153,12 +3153,12 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>alle-wierook</t>
+          <t>witte-salie-en-smudges</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>palo-santo-alle-producten</t>
+          <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
@@ -3216,7 +3216,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>zoutlampen-en-meer</t>
+          <t>mineralen-decoratie-producten</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
@@ -3247,12 +3247,12 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>banners-wandkleden-en-strandlakens</t>
+          <t>alle-beelden</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>klein-meubilair-en-decoratie</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -3319,12 +3319,12 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>alle-sieraden</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>malas-en-mala-tasjes</t>
+          <t>sieraden-accessoires</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
@@ -3355,12 +3355,12 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>stemvorken</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>alle-metalen-klankschalen</t>
+          <t>accessoires-metalen-klankschalen</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
@@ -3391,12 +3391,12 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>alle-metalen-klankschalen</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>sound-healing-instrumenten</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>alle-metalen-klankschalen</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -3463,12 +3463,12 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>alle-metalen-klankschalen</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>sound-healing-instrumenten</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
@@ -3499,12 +3499,12 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>alle-metalen-klankschalen</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>sound-healing-instrumenten</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr">
@@ -3557,12 +3557,12 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>alle-metalen-klankschalen</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>sound-healing-instrumenten</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
@@ -3593,12 +3593,12 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>alle-metalen-klankschalen</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>sound-healing-instrumenten</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr">
@@ -3629,12 +3629,12 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>alle-metalen-klankschalen</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>sound-healing-instrumenten</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr">
@@ -3665,12 +3665,12 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>alle-metalen-klankschalen</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>sound-healing-instrumenten</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
@@ -3701,12 +3701,12 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>alle-metalen-klankschalen</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>sound-healing-instrumenten</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="H96" s="2" t="inlineStr">
@@ -3737,12 +3737,12 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>alle-metalen-klankschalen</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>sound-healing-instrumenten</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr">
@@ -3773,12 +3773,12 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>alle-metalen-klankschalen</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>sound-healing-instrumenten</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr">
@@ -3809,12 +3809,12 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>alle-metalen-klankschalen</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>sound-healing-instrumenten</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr">
@@ -3845,12 +3845,12 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>alle-metalen-klankschalen</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>sound-healing-instrumenten</t>
+          <t>tibetaanse-wierook</t>
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr">
@@ -3881,12 +3881,12 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>alle-metalen-klankschalen</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>sound-healing-instrumenten</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="H101" s="2" t="inlineStr">
@@ -3922,7 +3922,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>kamerfonteinen</t>
+          <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
       <c r="H102" s="2" t="inlineStr">
@@ -3953,12 +3953,12 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>alle-kristallen-klankschalen</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>sound-healing-instrumenten</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="H103" s="2" t="inlineStr">
@@ -3989,12 +3989,12 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>alle-kristallen-klankschalen</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>sound-healing-instrumenten</t>
+          <t>chakra-producten</t>
         </is>
       </c>
       <c r="H104" s="2" t="inlineStr">
@@ -4025,12 +4025,12 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>alle-kristallen-klankschalen</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>sound-healing-instrumenten</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="H105" s="2" t="inlineStr">
@@ -4061,12 +4061,12 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>alle-kristallen-klankschalen</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>sound-healing-instrumenten</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="H106" s="2" t="inlineStr">
@@ -4102,7 +4102,7 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>biologische-ontspanningsproducten</t>
+          <t>massageolie</t>
         </is>
       </c>
       <c r="H107" s="2" t="inlineStr">
@@ -4241,12 +4241,12 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>biologische-lichaamsverzorging</t>
+          <t>gezichtsverzorging</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>gezichtsverzorging</t>
+          <t>haarverzorging</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -4299,12 +4299,12 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>sfeerlichten-en-lantaarns</t>
+          <t>waxinelichtjes</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>waxinelichtjes</t>
+          <t>klein-meubilair-en-decoratie</t>
         </is>
       </c>
       <c r="H113" s="2" t="inlineStr">
@@ -4423,12 +4423,12 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>kettingen-en-malas</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>alle-sieraden</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="H117" s="2" t="inlineStr">
@@ -4459,12 +4459,12 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>alle-kaarsen</t>
+          <t>wicca-en-tarot</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>wicca-en-tarot</t>
+          <t>witte-salie-en-smudges</t>
         </is>
       </c>
       <c r="H118" s="2" t="inlineStr">
@@ -4495,12 +4495,12 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>alle-wierook</t>
+          <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>nag-champa-en-satya-wierook</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="H119" s="2" t="inlineStr">
@@ -4536,7 +4536,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>lichaamsverzorging-producten</t>
+          <t>biologische-ontspanningsproducten</t>
         </is>
       </c>
       <c r="H120" s="2" t="inlineStr">
@@ -4567,12 +4567,12 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
+          <t>biologische-ontspanningsproducten</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
           <t>lichaamsverzorging-producten</t>
-        </is>
-      </c>
-      <c r="G121" t="inlineStr">
-        <is>
-          <t>biologische-ontspanningsproducten</t>
         </is>
       </c>
       <c r="H121" s="2" t="inlineStr">
@@ -4625,7 +4625,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>watervitalisering-natures-design</t>
+          <t>watervitalisering-edelsteenstaven</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
@@ -4661,12 +4661,12 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>meditatiebankjes</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>sjaals-en-pashminas</t>
+          <t>alle-metalen-klankschalen</t>
         </is>
       </c>
       <c r="H124" s="2" t="inlineStr">
@@ -4697,12 +4697,12 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>alle-meditatiekussens</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>meditatiematten-en-meditatiesets</t>
+          <t>alle-metalen-klankschalen</t>
         </is>
       </c>
       <c r="H125" s="2" t="inlineStr">
@@ -4733,12 +4733,12 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>alle-meditatiekussens</t>
+          <t>chakra-producten</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>chakra-producten</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="H126" s="2" t="inlineStr">
@@ -4769,12 +4769,12 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>alle-meditatiekussens</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>meditatiekussens-rond</t>
+          <t>alle-metalen-klankschalen</t>
         </is>
       </c>
       <c r="H127" s="2" t="inlineStr">
@@ -4805,12 +4805,12 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>alle-meditatiekussens</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>meditatiekussens-rond-biologisch</t>
+          <t>alle-metalen-klankschalen</t>
         </is>
       </c>
       <c r="H128" s="2" t="inlineStr">
@@ -4841,12 +4841,12 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>biologische-meditatiekussens</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>alle-meditatiekussens</t>
+          <t>alle-metalen-klankschalen</t>
         </is>
       </c>
       <c r="H129" s="2" t="inlineStr">
@@ -4877,12 +4877,12 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>alle-meditatiekussens</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>meditatiebankjes</t>
+          <t>alle-metalen-klankschalen</t>
         </is>
       </c>
       <c r="H130" s="2" t="inlineStr">
@@ -4918,7 +4918,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>zorgenstenen-en-knuffelstenen</t>
+          <t>biologische-ontspanningsproducten</t>
         </is>
       </c>
       <c r="H131" s="2" t="inlineStr">
@@ -4949,12 +4949,12 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>edelsteen-bollen</t>
+          <t>seleniet-producten</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>edelsteen-piramides-obelisk</t>
+          <t>klein-meubilair-en-decoratie</t>
         </is>
       </c>
       <c r="H132" s="2" t="inlineStr">
@@ -5007,12 +5007,12 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>alle-wierook</t>
+          <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>masala-en-ayurvedische-wierook</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="H134" s="2" t="inlineStr">
@@ -5043,12 +5043,12 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>lichaamsverzorging-producten</t>
+          <t>haarverzorging</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>biologische-lichaamsverzorging</t>
+          <t>gezichtsverzorging</t>
         </is>
       </c>
       <c r="H135" s="2" t="inlineStr">
@@ -5105,12 +5105,12 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>alle-wierook</t>
+          <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>masala-en-ayurvedische-wierook</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="H137" s="2" t="n"/>
@@ -5209,12 +5209,12 @@
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>alle-sieraden</t>
+          <t>sieraden-accessoires</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>edelsteen-oorbellen</t>
+          <t>verpakkingen-potjes-dozen-tasjes</t>
         </is>
       </c>
       <c r="H140" s="2" t="inlineStr">
@@ -5245,12 +5245,12 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>alle-kaarsen</t>
+          <t>biologische-ontspanningsproducten</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>biologische-ontspanningsproducten</t>
+          <t>massage-hulpmiddelen</t>
         </is>
       </c>
       <c r="H141" s="2" t="inlineStr">
@@ -5281,12 +5281,12 @@
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>shungiet-producten</t>
+          <t>feng-shui-kristalproducten</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>feng-shui-kristalproducten</t>
+          <t>seleniet-producten</t>
         </is>
       </c>
       <c r="H142" s="2" t="inlineStr">
@@ -5322,7 +5322,7 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>kamerfonteinen</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="H143" s="2" t="inlineStr">
@@ -5353,12 +5353,12 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>palo-santo-wierook</t>
+          <t>witte-salie-en-smudges</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>palo-santo-sieraden</t>
+          <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
       <c r="H144" s="2" t="inlineStr">
@@ -5394,7 +5394,7 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>alle-sieraden</t>
+          <t>verpakkingen-potjes-dozen-tasjes</t>
         </is>
       </c>
       <c r="H145" s="2" t="inlineStr">
@@ -5425,12 +5425,12 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>palo-santo-alle-producten</t>
+          <t>witte-salie-en-smudges</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>alle-wierook</t>
+          <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
       <c r="H146" s="2" t="n"/>
@@ -5457,12 +5457,12 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>interieur-geurproducten</t>
+          <t>gezichtsverzorging</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>gezichtsverzorging</t>
+          <t>bad-douche-en-zeep</t>
         </is>
       </c>
       <c r="H147" s="2" t="inlineStr">
@@ -5529,12 +5529,12 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>pendels-voor-professionals</t>
+          <t>biotensors-en-wichelroedes</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>biotensors-en-wichelroedes</t>
+          <t>wicca-en-tarot</t>
         </is>
       </c>
       <c r="H149" s="2" t="inlineStr">
@@ -5565,12 +5565,12 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>pendels-van-mineralen-hout-en-rudraksha</t>
+          <t>biotensors-en-wichelroedes</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>biotensors-en-wichelroedes</t>
+          <t>wicca-en-tarot</t>
         </is>
       </c>
       <c r="H150" s="2" t="inlineStr">
@@ -5668,7 +5668,7 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>postkaarten</t>
+          <t>notitieboeken-en-meer</t>
         </is>
       </c>
       <c r="H153" s="2" t="inlineStr">
@@ -5699,12 +5699,12 @@
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>alle-sieraden</t>
+          <t>sieraden-accessoires</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>edelsteen-ringen</t>
+          <t>verpakkingen-potjes-dozen-tasjes</t>
         </is>
       </c>
       <c r="H154" s="2" t="inlineStr">
@@ -5771,12 +5771,12 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>trommelstenen</t>
+          <t>seleniet-producten</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>mineralen-decoratie-producten</t>
+          <t>witte-salie-en-smudges</t>
         </is>
       </c>
       <c r="H156" s="2" t="inlineStr">
@@ -5807,12 +5807,12 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>trommelstenen</t>
+          <t>seleniet-producten</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>ruwe-edelstenen-power-boxen</t>
+          <t>witte-salie-en-smudges</t>
         </is>
       </c>
       <c r="H157" s="2" t="inlineStr">
@@ -5843,12 +5843,12 @@
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>alle-wierook</t>
+          <t>witte-salie-en-smudges</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>witte-salie-en-smudges</t>
+          <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
       <c r="H158" s="2" t="n"/>
@@ -5911,12 +5911,12 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>mineralen-decoratie-producten</t>
+          <t>trommelstenen</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>zoutlampen-en-meer</t>
+          <t>ruwe-onbewerkte-mineralen</t>
         </is>
       </c>
       <c r="H160" s="2" t="inlineStr">
@@ -5973,12 +5973,12 @@
       </c>
       <c r="F162" t="inlineStr">
         <is>
+          <t>waxinelichtjes</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
           <t>geurkaarsen</t>
-        </is>
-      </c>
-      <c r="G162" t="inlineStr">
-        <is>
-          <t>waxinelichtjes</t>
         </is>
       </c>
       <c r="H162" s="2" t="inlineStr">
@@ -6009,12 +6009,12 @@
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>orgoniet-producten</t>
+          <t>seleniet-producten</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>ruwe-onbewerkte-mineralen</t>
+          <t>watervitalisering-alle-producten</t>
         </is>
       </c>
       <c r="H163" s="2" t="inlineStr">
@@ -6067,12 +6067,12 @@
       </c>
       <c r="F165" t="inlineStr">
         <is>
+          <t>verpakkingen-potjes-dozen-tasjes</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
           <t>sieraden-opbergdozen-en-tasjes</t>
-        </is>
-      </c>
-      <c r="G165" t="inlineStr">
-        <is>
-          <t>edelsteen-armbanden</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -6108,7 +6108,7 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>alle-sieraden</t>
+          <t>verpakkingen-potjes-dozen-tasjes</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -6139,12 +6139,12 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>alle-sieraden</t>
+          <t>sieraden-accessoires</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>oorbellen</t>
+          <t>verpakkingen-potjes-dozen-tasjes</t>
         </is>
       </c>
       <c r="H167" s="2" t="inlineStr">
@@ -6180,7 +6180,7 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>alle-sieraden</t>
+          <t>verpakkingen-potjes-dozen-tasjes</t>
         </is>
       </c>
       <c r="H168" s="2" t="inlineStr">
@@ -6216,7 +6216,7 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>alle-sieraden</t>
+          <t>verpakkingen-potjes-dozen-tasjes</t>
         </is>
       </c>
       <c r="H169" s="2" t="inlineStr">
@@ -6247,12 +6247,12 @@
       </c>
       <c r="F170" t="inlineStr">
         <is>
+          <t>sieraden-accessoires</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
           <t>verpakkingen-potjes-dozen-tasjes</t>
-        </is>
-      </c>
-      <c r="G170" t="inlineStr">
-        <is>
-          <t>tassen-en-tasjes</t>
         </is>
       </c>
       <c r="H170" s="2" t="inlineStr">
@@ -6283,12 +6283,12 @@
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>meditatie-omslagdoeken-en-accessoires</t>
+          <t>alle-sieraden</t>
         </is>
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>yoga-omslagdoeken</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="H171" s="2" t="inlineStr">
@@ -6319,12 +6319,12 @@
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>alle-etherische-olien</t>
+          <t>aroma-diffusers</t>
         </is>
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>song-of-india-r-expo-wierook</t>
+          <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
       <c r="H172" s="2" t="inlineStr">
@@ -6355,12 +6355,12 @@
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>song-of-india-r-expo-wierook</t>
+          <t>olieverdampers-en-geurstenen</t>
         </is>
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>song-of-india-essentiele-olien</t>
+          <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
       <c r="H173" s="2" t="inlineStr">
@@ -6391,12 +6391,12 @@
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>alle-wierook</t>
+          <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>song-of-india-essentiele-olien</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="H174" s="2" t="n"/>
@@ -6423,12 +6423,12 @@
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>alle-metalen-klankschalen</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>gongs-gongtassen-en-gongstandaards</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="H175" s="2" t="inlineStr">
@@ -6525,12 +6525,12 @@
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>klankbuizen-en-klankstaven</t>
+          <t>trommelstenen</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>alle-metalen-klankschalen</t>
+          <t>chakra-producten</t>
         </is>
       </c>
       <c r="H179" s="2" t="inlineStr">
@@ -6566,7 +6566,7 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>postkaarten</t>
+          <t>notitieboeken-en-meer</t>
         </is>
       </c>
       <c r="H180" s="2" t="inlineStr">
@@ -6638,7 +6638,7 @@
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>malas-en-mala-tasjes</t>
+          <t>alle-sieraden</t>
         </is>
       </c>
       <c r="H182" s="2" t="inlineStr">
@@ -6718,7 +6718,7 @@
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>thee-shoti-maa-biologisch</t>
+          <t>geurkaarsen</t>
         </is>
       </c>
       <c r="H185" s="2" t="inlineStr">
@@ -6749,12 +6749,12 @@
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>biologische-thee</t>
+          <t>biologische-ontspanningsproducten</t>
         </is>
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>thee-shoti-maa-biologisch</t>
+          <t>geurkaarsen</t>
         </is>
       </c>
       <c r="H186" s="2" t="inlineStr">
@@ -6785,12 +6785,12 @@
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>thee-alle-producten</t>
+          <t>biologische-ontspanningsproducten</t>
         </is>
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>biologische-thee</t>
+          <t>geurkaarsen</t>
         </is>
       </c>
       <c r="H187" s="2" t="inlineStr">
@@ -6821,12 +6821,12 @@
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>thee-alle-producten</t>
+          <t>biologische-ontspanningsproducten</t>
         </is>
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>biologische-thee</t>
+          <t>geurkaarsen</t>
         </is>
       </c>
       <c r="H188" s="2" t="inlineStr">
@@ -6857,12 +6857,12 @@
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>thee-alle-producten</t>
+          <t>biologische-ontspanningsproducten</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>biologische-thee</t>
+          <t>geurkaarsen</t>
         </is>
       </c>
       <c r="H189" s="2" t="inlineStr">
@@ -6893,12 +6893,12 @@
       </c>
       <c r="F190" t="inlineStr">
         <is>
+          <t>tibetaanse-wierook</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
           <t>banners-wandkleden-en-strandlakens</t>
-        </is>
-      </c>
-      <c r="G190" t="inlineStr">
-        <is>
-          <t>tibetaanse-wierook</t>
         </is>
       </c>
       <c r="H190" s="2" t="inlineStr">
@@ -6965,12 +6965,12 @@
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>alle-wierook</t>
+          <t>tibetaanse-producten</t>
         </is>
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>tibetaanse-producten</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="H192" s="2" t="n"/>
@@ -6997,12 +6997,12 @@
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>trommelstenen-mini-chips</t>
+          <t>seleniet-producten</t>
         </is>
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>ruwe-onbewerkte-mineralen</t>
+          <t>sieraden-opbergdozen-en-tasjes</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -7033,12 +7033,12 @@
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>zorgenstenen-en-knuffelstenen</t>
+          <t>verpakkingen-potjes-dozen-tasjes</t>
         </is>
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>ruwe-onbewerkte-mineralen</t>
+          <t>seleniet-producten</t>
         </is>
       </c>
       <c r="H194" s="2" t="inlineStr">
@@ -7136,7 +7136,7 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>notitieboeken-en-meer</t>
+          <t>postkaarten</t>
         </is>
       </c>
       <c r="H197" s="2" t="inlineStr">
@@ -7167,12 +7167,12 @@
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>alle-kaarsen</t>
+          <t>zoutkristal-kaarshouders</t>
         </is>
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>honderd-uur-kaarsen</t>
+          <t>klein-meubilair-en-decoratie</t>
         </is>
       </c>
       <c r="H198" s="2" t="inlineStr">
@@ -7203,12 +7203,12 @@
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>watervitalisering-vitajuwel</t>
+          <t>watervitalisering-edelsteenstaven</t>
         </is>
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>watervitalisering-natures-design</t>
+          <t>watervitalisering-mineraalstaven</t>
         </is>
       </c>
       <c r="H199" s="2" t="inlineStr">
@@ -7239,12 +7239,12 @@
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>watervitalisering-mineraalstaven</t>
+          <t>meditatie-drinkflessen</t>
         </is>
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>meditatie-drinkflessen</t>
+          <t>watervitalisering-vitajuwel</t>
         </is>
       </c>
       <c r="H200" s="2" t="inlineStr">
@@ -7275,12 +7275,12 @@
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>watervitalisering-edelsteenstaven</t>
+          <t>meditatie-drinkflessen</t>
         </is>
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>meditatie-drinkflessen</t>
+          <t>watervitalisering-natures-design</t>
         </is>
       </c>
       <c r="H201" s="2" t="inlineStr">
@@ -7311,12 +7311,12 @@
       </c>
       <c r="F202" t="inlineStr">
         <is>
+          <t>watervitalisering-edelsteenstaven</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
           <t>meditatie-drinkflessen</t>
-        </is>
-      </c>
-      <c r="G202" t="inlineStr">
-        <is>
-          <t>watervitalisering-vitajuwel</t>
         </is>
       </c>
       <c r="H202" s="2" t="inlineStr">
@@ -7352,7 +7352,7 @@
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>watervitalisering-natures-design</t>
+          <t>watervitalisering-edelsteenstaven</t>
         </is>
       </c>
       <c r="H203" s="2" t="inlineStr">
@@ -7388,7 +7388,7 @@
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>alle-kaarsen</t>
+          <t>zoutlampen-en-meer</t>
         </is>
       </c>
       <c r="H204" s="2" t="inlineStr">
@@ -7424,7 +7424,7 @@
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>chakra-en-wicca-mineraalsets</t>
+          <t>manifestatiekaarsen</t>
         </is>
       </c>
       <c r="H205" s="2" t="inlineStr">
@@ -7477,7 +7477,7 @@
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>alle-wierook</t>
+          <t>wierookhouders-en-accessoires</t>
         </is>
       </c>
       <c r="G207" t="inlineStr">
@@ -7549,12 +7549,12 @@
       </c>
       <c r="F209" t="inlineStr">
         <is>
-          <t>alle-wierook</t>
+          <t>sfeerlichten-en-lantaarns</t>
         </is>
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>backflow-branders-kegels</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="H209" s="2" t="n"/>
@@ -7617,12 +7617,12 @@
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>wierookharsen-en-wierookkruiden</t>
+          <t>rituele-voorwerpen</t>
         </is>
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t>rituele-voorwerpen</t>
+          <t>ruwe-onbewerkte-mineralen</t>
         </is>
       </c>
       <c r="H211" s="2" t="inlineStr">
@@ -7716,7 +7716,7 @@
       </c>
       <c r="G214" t="inlineStr">
         <is>
-          <t>sjaals-en-pashminas</t>
+          <t>yoga-wierook</t>
         </is>
       </c>
       <c r="H214" s="2" t="inlineStr">
@@ -7783,12 +7783,12 @@
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t>biologische-yogaproducten</t>
+          <t>yoga-wierook</t>
         </is>
       </c>
       <c r="G216" t="inlineStr">
         <is>
-          <t>yoga-wierook</t>
+          <t>yogariemen-en-yogawiel</t>
         </is>
       </c>
       <c r="H216" s="2" t="inlineStr">
@@ -7819,12 +7819,12 @@
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t>alle-wierook</t>
+          <t>yoga-welzijn</t>
         </is>
       </c>
       <c r="G217" t="inlineStr">
         <is>
-          <t>yoga-welzijn</t>
+          <t>alle-meditatiekussens</t>
         </is>
       </c>
       <c r="H217" s="2" t="n"/>
@@ -7887,7 +7887,7 @@
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t>biologische-yogaproducten</t>
+          <t>yogariemen-en-yogawiel</t>
         </is>
       </c>
       <c r="G219" t="inlineStr">
@@ -7959,12 +7959,12 @@
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t>klein-meubilair-en-decoratie</t>
+          <t>alle-wierook</t>
         </is>
       </c>
       <c r="G221" t="inlineStr">
         <is>
-          <t>backflow-branders-kegels</t>
+          <t>wierookkegels</t>
         </is>
       </c>
       <c r="H221" s="2" t="inlineStr">
@@ -7995,12 +7995,12 @@
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>trommelstenen-mini-chips</t>
+          <t>sieraden-opbergdozen-en-tasjes</t>
         </is>
       </c>
       <c r="G222" t="inlineStr">
         <is>
-          <t>ruwe-onbewerkte-mineralen</t>
+          <t>witte-salie-en-smudges</t>
         </is>
       </c>
       <c r="H222" s="2" t="inlineStr">
@@ -8031,12 +8031,12 @@
       </c>
       <c r="F223" t="inlineStr">
         <is>
+          <t>alle-kaarsen</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
           <t>sfeerlichten-en-lantaarns</t>
-        </is>
-      </c>
-      <c r="G223" t="inlineStr">
-        <is>
-          <t>zoutlampen-en-meer</t>
         </is>
       </c>
       <c r="H223" s="2" t="inlineStr">
@@ -8067,7 +8067,7 @@
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t>zoutkristal-kaarshouders</t>
+          <t>waxinelichtjes</t>
         </is>
       </c>
       <c r="G224" t="inlineStr">

</xml_diff>